<commit_message>
New audit-workspace plugin; version bumps; chrome-bridge as download
- audit-workspace (1.1.0): new skills audit-workspace-setup + caseware-crosswalk,
  bundled with trial-balance-prep + writing-styles; trial-balance-prep no longer standalone
- fs-review 2.1.0 (4 skills -> 1 orchestrator); suralink-binder + cch-axcess-suite 1.1.0
- chrome-bridge.zip + handouts/ added at repo root; CHANGELOG.md added

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/cch-axcess-suite/skills/cch-axcess/references/data/binder-program-template-nonprofit.xlsx
+++ b/cch-axcess-suite/skills/cch-axcess/references/data/binder-program-template-nonprofit.xlsx
@@ -433,7 +433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H152"/>
+  <dimension ref="A1:H169"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -467,7 +467,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
@@ -2109,12 +2108,12 @@
     <row r="60">
       <c r="A60" s="3" t="inlineStr">
         <is>
-          <t>0606</t>
+          <t>0605.1</t>
         </is>
       </c>
       <c r="B60" s="3" t="inlineStr">
         <is>
-          <t>AUD-901 Audit Program Subsequent Events</t>
+          <t>AUD-818 Audit Program Fair Value Measurements and Disclosures</t>
         </is>
       </c>
       <c r="C60" s="3" t="inlineStr">
@@ -2124,31 +2123,39 @@
       </c>
       <c r="D60" s="3" t="inlineStr">
         <is>
-          <t>Subsequent events procedures</t>
+          <t>Fair value measurements and disclosures procedures</t>
         </is>
       </c>
       <c r="E60" s="3" t="inlineStr">
         <is>
-          <t>0601 near complete</t>
-        </is>
-      </c>
-      <c r="F60" s="3" t="n"/>
-      <c r="G60" s="3" t="inlineStr"/>
+          <t>0500</t>
+        </is>
+      </c>
+      <c r="F60" s="3" t="inlineStr">
+        <is>
+          <t>TB-driven overlay — add when FV measurements/disclosures exist (investments, split-interest, in-kind)</t>
+        </is>
+      </c>
+      <c r="G60" s="3" t="inlineStr">
+        <is>
+          <t>if-fair-value</t>
+        </is>
+      </c>
       <c r="H60" s="3" t="inlineStr">
         <is>
-          <t>AUD-901</t>
+          <t>—</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="3" t="inlineStr">
         <is>
-          <t>0607</t>
+          <t>0605.2</t>
         </is>
       </c>
       <c r="B61" s="3" t="inlineStr">
         <is>
-          <t>KBA-902 Audit Review and Approval Checklist</t>
+          <t>AUD-819 Audit Program Commitments and Contingencies</t>
         </is>
       </c>
       <c r="C61" s="3" t="inlineStr">
@@ -2158,31 +2165,39 @@
       </c>
       <c r="D61" s="3" t="inlineStr">
         <is>
-          <t>Partner/manager review sign-off checklist</t>
+          <t>Commitments and contingencies procedures</t>
         </is>
       </c>
       <c r="E61" s="3" t="inlineStr">
         <is>
-          <t>0601</t>
-        </is>
-      </c>
-      <c r="F61" s="3" t="n"/>
-      <c r="G61" s="3" t="inlineStr"/>
+          <t>0300, 0500</t>
+        </is>
+      </c>
+      <c r="F61" s="3" t="inlineStr">
+        <is>
+          <t>TB-driven overlay — add when leases, conditional grants, litigation, or other commitments exist</t>
+        </is>
+      </c>
+      <c r="G61" s="3" t="inlineStr">
+        <is>
+          <t>if-commitments</t>
+        </is>
+      </c>
       <c r="H61" s="3" t="inlineStr">
         <is>
-          <t>KBA-902</t>
+          <t>—</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="3" t="inlineStr">
         <is>
-          <t>0608</t>
+          <t>0605.3</t>
         </is>
       </c>
       <c r="B62" s="3" t="inlineStr">
         <is>
-          <t>KBA-904 Audit Documentation Checklist</t>
+          <t>AUD-820 Audit Program Accounting Estimate</t>
         </is>
       </c>
       <c r="C62" s="3" t="inlineStr">
@@ -2192,31 +2207,39 @@
       </c>
       <c r="D62" s="3" t="inlineStr">
         <is>
-          <t>FS audit file assembly and documentation completeness checklist</t>
+          <t>Accounting estimates procedures; pairs with KBA-105 at 0600</t>
         </is>
       </c>
       <c r="E62" s="3" t="inlineStr">
         <is>
-          <t>0607</t>
-        </is>
-      </c>
-      <c r="F62" s="3" t="n"/>
-      <c r="G62" s="3" t="inlineStr"/>
+          <t>0500, 0600</t>
+        </is>
+      </c>
+      <c r="F62" s="3" t="inlineStr">
+        <is>
+          <t>TB-driven overlay — add when significant estimates exist (allowances, useful lives, accruals)</t>
+        </is>
+      </c>
+      <c r="G62" s="3" t="inlineStr">
+        <is>
+          <t>if-estimates</t>
+        </is>
+      </c>
       <c r="H62" s="3" t="inlineStr">
         <is>
-          <t>KBA-903</t>
+          <t>—</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="3" t="inlineStr">
         <is>
-          <t>0608.1</t>
+          <t>0605.4</t>
         </is>
       </c>
       <c r="B63" s="3" t="inlineStr">
         <is>
-          <t>KBA-903S Compliance Audit Documentation Checklist</t>
+          <t>AUD-821 Audit Program Concentrations</t>
         </is>
       </c>
       <c r="C63" s="3" t="inlineStr">
@@ -2226,101 +2249,173 @@
       </c>
       <c r="D63" s="3" t="inlineStr">
         <is>
-          <t>SA audit file assembly and documentation completeness checklist; parallel to KBA-903</t>
+          <t>Concentrations procedures</t>
         </is>
       </c>
       <c r="E63" s="3" t="inlineStr">
         <is>
-          <t>0608, 8110</t>
+          <t>0300, 0500</t>
         </is>
       </c>
       <c r="F63" s="3" t="inlineStr">
         <is>
-          <t>Complete after all SA programs done; references AUD-100S</t>
+          <t>TB-driven overlay — add when donor/grantor/vendor/deposit concentrations exist</t>
         </is>
       </c>
       <c r="G63" s="3" t="inlineStr">
         <is>
-          <t>if-single-audit</t>
+          <t>if-concentrations</t>
         </is>
       </c>
       <c r="H63" s="3" t="inlineStr">
         <is>
-          <t>KBA-903S</t>
+          <t>—</t>
         </is>
       </c>
     </row>
     <row r="64">
-      <c r="A64" s="3" t="n"/>
-      <c r="B64" s="3" t="n"/>
-      <c r="C64" s="3" t="n"/>
-      <c r="D64" s="3" t="n"/>
-      <c r="E64" s="3" t="n"/>
+      <c r="A64" s="3" t="inlineStr">
+        <is>
+          <t>0606</t>
+        </is>
+      </c>
+      <c r="B64" s="3" t="inlineStr">
+        <is>
+          <t>AUD-901 Audit Program Subsequent Events</t>
+        </is>
+      </c>
+      <c r="C64" s="3" t="inlineStr">
+        <is>
+          <t>KC Form</t>
+        </is>
+      </c>
+      <c r="D64" s="3" t="inlineStr">
+        <is>
+          <t>Subsequent events procedures</t>
+        </is>
+      </c>
+      <c r="E64" s="3" t="inlineStr">
+        <is>
+          <t>0601 near complete</t>
+        </is>
+      </c>
       <c r="F64" s="3" t="n"/>
-      <c r="G64" s="3" t="n"/>
-      <c r="H64" s="3" t="n"/>
+      <c r="G64" s="3" t="inlineStr"/>
+      <c r="H64" s="3" t="inlineStr">
+        <is>
+          <t>AUD-901</t>
+        </is>
+      </c>
     </row>
     <row r="65">
-      <c r="A65" s="2" t="inlineStr">
-        <is>
-          <t>SECTION 07 — REPORTS AND COMMUNICATIONS AT THE CONCLUSION OF AN AUDIT</t>
-        </is>
-      </c>
-      <c r="B65" s="3" t="n"/>
-      <c r="C65" s="3" t="n"/>
-      <c r="D65" s="3" t="n"/>
-      <c r="E65" s="3" t="n"/>
+      <c r="A65" s="3" t="inlineStr">
+        <is>
+          <t>0607</t>
+        </is>
+      </c>
+      <c r="B65" s="3" t="inlineStr">
+        <is>
+          <t>KBA-902 Audit Review and Approval Checklist</t>
+        </is>
+      </c>
+      <c r="C65" s="3" t="inlineStr">
+        <is>
+          <t>KC Form</t>
+        </is>
+      </c>
+      <c r="D65" s="3" t="inlineStr">
+        <is>
+          <t>Partner/manager review sign-off checklist</t>
+        </is>
+      </c>
+      <c r="E65" s="3" t="inlineStr">
+        <is>
+          <t>0601</t>
+        </is>
+      </c>
       <c r="F65" s="3" t="n"/>
-      <c r="G65" s="3" t="n"/>
-      <c r="H65" s="3" t="n"/>
+      <c r="G65" s="3" t="inlineStr"/>
+      <c r="H65" s="3" t="inlineStr">
+        <is>
+          <t>KBA-902</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="3" t="inlineStr">
         <is>
-          <t>0700</t>
+          <t>0608</t>
         </is>
       </c>
       <c r="B66" s="3" t="inlineStr">
         <is>
-          <t>Financial Statements</t>
+          <t>KBA-904 Audit Documentation Checklist</t>
         </is>
       </c>
       <c r="C66" s="3" t="inlineStr">
         <is>
-          <t>Client Doc</t>
+          <t>KC Form</t>
         </is>
       </c>
       <c r="D66" s="3" t="inlineStr">
         <is>
-          <t>Audited financial statements</t>
+          <t>FS audit file assembly and documentation completeness checklist</t>
         </is>
       </c>
       <c r="E66" s="3" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F66" s="3" t="inlineStr">
-        <is>
-          <t>Moved from front of file; filed here with final reports</t>
-        </is>
-      </c>
+          <t>0607</t>
+        </is>
+      </c>
+      <c r="F66" s="3" t="n"/>
       <c r="G66" s="3" t="inlineStr"/>
-      <c r="H66" s="3" t="inlineStr"/>
+      <c r="H66" s="3" t="inlineStr">
+        <is>
+          <t>KBA-903</t>
+        </is>
+      </c>
     </row>
     <row r="67">
-      <c r="A67" s="3" t="n"/>
+      <c r="A67" s="3" t="inlineStr">
+        <is>
+          <t>0608.1</t>
+        </is>
+      </c>
       <c r="B67" s="3" t="inlineStr">
         <is>
-          <t>Whatever other letters, MLCs, SAS 114/115, powerpoint presentations, etc.</t>
-        </is>
-      </c>
-      <c r="C67" s="3" t="n"/>
-      <c r="D67" s="3" t="n"/>
-      <c r="E67" s="3" t="n"/>
-      <c r="F67" s="3" t="n"/>
-      <c r="G67" s="3" t="inlineStr"/>
-      <c r="H67" s="3" t="inlineStr"/>
+          <t>KBA-903S Compliance Audit Documentation Checklist</t>
+        </is>
+      </c>
+      <c r="C67" s="3" t="inlineStr">
+        <is>
+          <t>KC Form</t>
+        </is>
+      </c>
+      <c r="D67" s="3" t="inlineStr">
+        <is>
+          <t>SA audit file assembly and documentation completeness checklist; parallel to KBA-903</t>
+        </is>
+      </c>
+      <c r="E67" s="3" t="inlineStr">
+        <is>
+          <t>0608, 8110</t>
+        </is>
+      </c>
+      <c r="F67" s="3" t="inlineStr">
+        <is>
+          <t>Complete after all SA programs done; references AUD-100S</t>
+        </is>
+      </c>
+      <c r="G67" s="3" t="inlineStr">
+        <is>
+          <t>if-single-audit</t>
+        </is>
+      </c>
+      <c r="H67" s="3" t="inlineStr">
+        <is>
+          <t>KBA-903S</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="3" t="n"/>
@@ -2335,7 +2430,7 @@
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
         <is>
-          <t>SECTION 09 — TRIAL BALANCE</t>
+          <t>SECTION 07 — REPORTS AND COMMUNICATIONS AT THE CONCLUSION OF AN AUDIT</t>
         </is>
       </c>
       <c r="B69" s="3" t="n"/>
@@ -2349,95 +2444,67 @@
     <row r="70">
       <c r="A70" s="3" t="inlineStr">
         <is>
-          <t>0900</t>
+          <t>0700</t>
         </is>
       </c>
       <c r="B70" s="3" t="inlineStr">
         <is>
-          <t>Trial Balance — Group Summary</t>
+          <t>Financial Statements</t>
         </is>
       </c>
       <c r="C70" s="3" t="inlineStr">
         <is>
-          <t>TB</t>
+          <t>Client Doc</t>
         </is>
       </c>
       <c r="D70" s="3" t="inlineStr">
         <is>
-          <t>Consolidated/group TB summary</t>
+          <t>Audited financial statements</t>
         </is>
       </c>
       <c r="E70" s="3" t="inlineStr">
         <is>
-          <t>Client</t>
-        </is>
-      </c>
-      <c r="F70" s="3" t="n"/>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F70" s="3" t="inlineStr">
+        <is>
+          <t>Moved from front of file; filed here with final reports</t>
+        </is>
+      </c>
       <c r="G70" s="3" t="inlineStr"/>
       <c r="H70" s="3" t="inlineStr"/>
     </row>
     <row r="71">
-      <c r="A71" s="3" t="inlineStr">
-        <is>
-          <t>0900.1</t>
-        </is>
-      </c>
+      <c r="A71" s="3" t="n"/>
       <c r="B71" s="3" t="inlineStr">
         <is>
-          <t>Trial Balance — Group and Subgroup Summary</t>
-        </is>
-      </c>
-      <c r="C71" s="3" t="inlineStr">
-        <is>
-          <t>TB</t>
-        </is>
-      </c>
-      <c r="D71" s="3" t="inlineStr">
-        <is>
-          <t>TB by fund/subgroup</t>
-        </is>
-      </c>
-      <c r="E71" s="3" t="inlineStr">
-        <is>
-          <t>Client</t>
-        </is>
-      </c>
+          <t>Whatever other letters, MLCs, SAS 114/115, powerpoint presentations, etc.</t>
+        </is>
+      </c>
+      <c r="C71" s="3" t="n"/>
+      <c r="D71" s="3" t="n"/>
+      <c r="E71" s="3" t="n"/>
       <c r="F71" s="3" t="n"/>
       <c r="G71" s="3" t="inlineStr"/>
       <c r="H71" s="3" t="inlineStr"/>
     </row>
     <row r="72">
-      <c r="A72" s="3" t="inlineStr">
-        <is>
-          <t>0900.2</t>
-        </is>
-      </c>
-      <c r="B72" s="3" t="inlineStr">
-        <is>
-          <t>Trial Balance — Detail</t>
-        </is>
-      </c>
-      <c r="C72" s="3" t="inlineStr">
-        <is>
-          <t>TB</t>
-        </is>
-      </c>
-      <c r="D72" s="3" t="inlineStr">
-        <is>
-          <t>Full detail TB</t>
-        </is>
-      </c>
-      <c r="E72" s="3" t="inlineStr">
-        <is>
-          <t>Client</t>
-        </is>
-      </c>
+      <c r="A72" s="3" t="n"/>
+      <c r="B72" s="3" t="n"/>
+      <c r="C72" s="3" t="n"/>
+      <c r="D72" s="3" t="n"/>
+      <c r="E72" s="3" t="n"/>
       <c r="F72" s="3" t="n"/>
-      <c r="G72" s="3" t="inlineStr"/>
-      <c r="H72" s="3" t="inlineStr"/>
+      <c r="G72" s="3" t="n"/>
+      <c r="H72" s="3" t="n"/>
     </row>
     <row r="73">
-      <c r="A73" s="3" t="n"/>
+      <c r="A73" s="2" t="inlineStr">
+        <is>
+          <t>SECTION 09 — TRIAL BALANCE</t>
+        </is>
+      </c>
       <c r="B73" s="3" t="n"/>
       <c r="C73" s="3" t="n"/>
       <c r="D73" s="3" t="n"/>
@@ -2447,82 +2514,94 @@
       <c r="H73" s="3" t="n"/>
     </row>
     <row r="74">
-      <c r="A74" s="2" t="inlineStr">
-        <is>
-          <t>SECTION 10 — CASH &amp; CASH EQUIVALENTS</t>
-        </is>
-      </c>
-      <c r="B74" s="3" t="n"/>
-      <c r="C74" s="3" t="n"/>
-      <c r="D74" s="3" t="n"/>
-      <c r="E74" s="3" t="n"/>
+      <c r="A74" s="3" t="inlineStr">
+        <is>
+          <t>0900</t>
+        </is>
+      </c>
+      <c r="B74" s="3" t="inlineStr">
+        <is>
+          <t>Trial Balance — Group Summary</t>
+        </is>
+      </c>
+      <c r="C74" s="3" t="inlineStr">
+        <is>
+          <t>TB</t>
+        </is>
+      </c>
+      <c r="D74" s="3" t="inlineStr">
+        <is>
+          <t>Consolidated/group TB summary</t>
+        </is>
+      </c>
+      <c r="E74" s="3" t="inlineStr">
+        <is>
+          <t>Client</t>
+        </is>
+      </c>
       <c r="F74" s="3" t="n"/>
-      <c r="G74" s="3" t="n"/>
-      <c r="H74" s="3" t="n"/>
+      <c r="G74" s="3" t="inlineStr"/>
+      <c r="H74" s="3" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" s="3" t="inlineStr">
         <is>
-          <t>1000</t>
+          <t>0900.1</t>
         </is>
       </c>
       <c r="B75" s="3" t="inlineStr">
         <is>
-          <t>Cash &amp; Equivalents Leadsheet</t>
+          <t>Trial Balance — Group and Subgroup Summary</t>
         </is>
       </c>
       <c r="C75" s="3" t="inlineStr">
         <is>
-          <t>Workpaper</t>
+          <t>TB</t>
         </is>
       </c>
       <c r="D75" s="3" t="inlineStr">
         <is>
-          <t>Leadsheet reconciling cash per TB to audit</t>
+          <t>TB by fund/subgroup</t>
         </is>
       </c>
       <c r="E75" s="3" t="inlineStr">
         <is>
-          <t>0900</t>
+          <t>Client</t>
         </is>
       </c>
       <c r="F75" s="3" t="n"/>
-      <c r="G75" s="3" t="n"/>
-      <c r="H75" s="3" t="n"/>
+      <c r="G75" s="3" t="inlineStr"/>
+      <c r="H75" s="3" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" s="3" t="inlineStr">
         <is>
-          <t>1000-PROG</t>
+          <t>0900.2</t>
         </is>
       </c>
       <c r="B76" s="3" t="inlineStr">
         <is>
-          <t>AUD-801 Audit Program Cash</t>
+          <t>Trial Balance — Detail</t>
         </is>
       </c>
       <c r="C76" s="3" t="inlineStr">
         <is>
-          <t>KC Form</t>
+          <t>TB</t>
         </is>
       </c>
       <c r="D76" s="3" t="inlineStr">
         <is>
-          <t>Audit program — cash</t>
+          <t>Full detail TB</t>
         </is>
       </c>
       <c r="E76" s="3" t="inlineStr">
         <is>
-          <t>0203, 0500</t>
+          <t>Client</t>
         </is>
       </c>
       <c r="F76" s="3" t="n"/>
-      <c r="G76" s="3" t="n"/>
-      <c r="H76" s="3" t="inlineStr">
-        <is>
-          <t>AUD-801</t>
-        </is>
-      </c>
+      <c r="G76" s="3" t="inlineStr"/>
+      <c r="H76" s="3" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" s="3" t="n"/>
@@ -2537,7 +2616,7 @@
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>SECTION 12 — RECEIVABLES</t>
+          <t>SECTION 10 — CASH &amp; CASH EQUIVALENTS</t>
         </is>
       </c>
       <c r="B78" s="3" t="n"/>
@@ -2551,12 +2630,12 @@
     <row r="79">
       <c r="A79" s="3" t="inlineStr">
         <is>
-          <t>1200</t>
+          <t>1000</t>
         </is>
       </c>
       <c r="B79" s="3" t="inlineStr">
         <is>
-          <t>Receivables, net Leadsheet</t>
+          <t>Cash &amp; Equivalents Leadsheet</t>
         </is>
       </c>
       <c r="C79" s="3" t="inlineStr">
@@ -2566,7 +2645,7 @@
       </c>
       <c r="D79" s="3" t="inlineStr">
         <is>
-          <t>Leadsheet — receivables</t>
+          <t>Leadsheet reconciling cash per TB to audit</t>
         </is>
       </c>
       <c r="E79" s="3" t="inlineStr">
@@ -2581,12 +2660,12 @@
     <row r="80">
       <c r="A80" s="3" t="inlineStr">
         <is>
-          <t>1200-PROG</t>
+          <t>1000-PROG</t>
         </is>
       </c>
       <c r="B80" s="3" t="inlineStr">
         <is>
-          <t>AUD-803 Audit Program Accounts Receivable and Revenues</t>
+          <t>AUD-801 Audit Program Cash</t>
         </is>
       </c>
       <c r="C80" s="3" t="inlineStr">
@@ -2596,7 +2675,7 @@
       </c>
       <c r="D80" s="3" t="inlineStr">
         <is>
-          <t>Audit program — receivables/nonexchange revenue</t>
+          <t>Audit program — cash</t>
         </is>
       </c>
       <c r="E80" s="3" t="inlineStr">
@@ -2608,7 +2687,7 @@
       <c r="G80" s="3" t="n"/>
       <c r="H80" s="3" t="inlineStr">
         <is>
-          <t>AUD-804</t>
+          <t>AUD-801</t>
         </is>
       </c>
     </row>
@@ -2625,7 +2704,7 @@
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>SECTION 14 — PREPAID EXPENSES</t>
+          <t>SECTION 11 — INVESTMENTS</t>
         </is>
       </c>
       <c r="B82" s="3" t="n"/>
@@ -2639,12 +2718,12 @@
     <row r="83">
       <c r="A83" s="3" t="inlineStr">
         <is>
-          <t>1400</t>
+          <t>1100</t>
         </is>
       </c>
       <c r="B83" s="3" t="inlineStr">
         <is>
-          <t>Prepaid Expenses Leadsheet</t>
+          <t>Investments Leadsheet</t>
         </is>
       </c>
       <c r="C83" s="3" t="inlineStr">
@@ -2654,7 +2733,7 @@
       </c>
       <c r="D83" s="3" t="inlineStr">
         <is>
-          <t>Leadsheet — prepaids</t>
+          <t>Leadsheet — investments</t>
         </is>
       </c>
       <c r="E83" s="3" t="inlineStr">
@@ -2662,19 +2741,27 @@
           <t>0900</t>
         </is>
       </c>
-      <c r="F83" s="3" t="n"/>
-      <c r="G83" s="3" t="n"/>
+      <c r="F83" s="3" t="inlineStr">
+        <is>
+          <t>Add when TB carries investments</t>
+        </is>
+      </c>
+      <c r="G83" s="3" t="inlineStr">
+        <is>
+          <t>if-investments</t>
+        </is>
+      </c>
       <c r="H83" s="3" t="n"/>
     </row>
     <row r="84">
       <c r="A84" s="3" t="inlineStr">
         <is>
-          <t>1400-PROG</t>
+          <t>1100-PROG</t>
         </is>
       </c>
       <c r="B84" s="3" t="inlineStr">
         <is>
-          <t>AUD-807 Audit Program Ppds, Dfrds, Coll Items, Oth Assets</t>
+          <t>AUD-802 Audit Program Investments Including Programmatic Inv</t>
         </is>
       </c>
       <c r="C84" s="3" t="inlineStr">
@@ -2684,7 +2771,7 @@
       </c>
       <c r="D84" s="3" t="inlineStr">
         <is>
-          <t>Audit program — prepaids</t>
+          <t>Audit program — investments incl. programmatic investments</t>
         </is>
       </c>
       <c r="E84" s="3" t="inlineStr">
@@ -2692,28 +2779,27 @@
           <t>0203, 0500</t>
         </is>
       </c>
-      <c r="F84" s="3" t="n"/>
-      <c r="G84" s="3" t="n"/>
+      <c r="F84" s="3" t="inlineStr">
+        <is>
+          <t>TB-driven — add when TB carries investments (KBA-400 scoping confirms)</t>
+        </is>
+      </c>
+      <c r="G84" s="3" t="inlineStr">
+        <is>
+          <t>if-investments</t>
+        </is>
+      </c>
       <c r="H84" s="3" t="inlineStr">
         <is>
-          <t>AUD-806</t>
-        </is>
-      </c>
-    </row>
-    <row r="85">
-      <c r="A85" s="3" t="n"/>
-      <c r="B85" s="3" t="n"/>
-      <c r="C85" s="3" t="n"/>
-      <c r="D85" s="3" t="n"/>
-      <c r="E85" s="3" t="n"/>
-      <c r="F85" s="3" t="n"/>
-      <c r="G85" s="3" t="n"/>
-      <c r="H85" s="3" t="n"/>
-    </row>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="85"/>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>SECTION 20 — PAYABLES</t>
+          <t>SECTION 12 — RECEIVABLES</t>
         </is>
       </c>
       <c r="B86" s="3" t="n"/>
@@ -2727,12 +2813,12 @@
     <row r="87">
       <c r="A87" s="3" t="inlineStr">
         <is>
-          <t>2000</t>
+          <t>1200</t>
         </is>
       </c>
       <c r="B87" s="3" t="inlineStr">
         <is>
-          <t>Payables Leadsheet</t>
+          <t>Receivables, net Leadsheet</t>
         </is>
       </c>
       <c r="C87" s="3" t="inlineStr">
@@ -2742,7 +2828,7 @@
       </c>
       <c r="D87" s="3" t="inlineStr">
         <is>
-          <t>Leadsheet — payables</t>
+          <t>Leadsheet — receivables</t>
         </is>
       </c>
       <c r="E87" s="3" t="inlineStr">
@@ -2757,12 +2843,12 @@
     <row r="88">
       <c r="A88" s="3" t="inlineStr">
         <is>
-          <t>2000-PROG</t>
+          <t>1200-PROG</t>
         </is>
       </c>
       <c r="B88" s="3" t="inlineStr">
         <is>
-          <t>AUD-810 Audit Program Accounts Payable and Purchases</t>
+          <t>AUD-803 Audit Program Accounts Receivable and Revenues</t>
         </is>
       </c>
       <c r="C88" s="3" t="inlineStr">
@@ -2772,7 +2858,7 @@
       </c>
       <c r="D88" s="3" t="inlineStr">
         <is>
-          <t>Audit program — AP</t>
+          <t>Audit program — receivables/nonexchange revenue</t>
         </is>
       </c>
       <c r="E88" s="3" t="inlineStr">
@@ -2784,42 +2870,26 @@
       <c r="G88" s="3" t="n"/>
       <c r="H88" s="3" t="inlineStr">
         <is>
-          <t>AUD-808</t>
+          <t>AUD-804</t>
         </is>
       </c>
     </row>
     <row r="89">
-      <c r="A89" s="3" t="inlineStr">
-        <is>
-          <t>2001</t>
-        </is>
-      </c>
-      <c r="B89" s="3" t="inlineStr">
-        <is>
-          <t>Search for Unrecorded Liabilities</t>
-        </is>
-      </c>
-      <c r="C89" s="3" t="inlineStr">
-        <is>
-          <t>Workpaper</t>
-        </is>
-      </c>
-      <c r="D89" s="3" t="inlineStr">
-        <is>
-          <t>SUL testing workpaper</t>
-        </is>
-      </c>
-      <c r="E89" s="3" t="inlineStr">
-        <is>
-          <t>2000-PROG</t>
-        </is>
-      </c>
+      <c r="A89" s="3" t="n"/>
+      <c r="B89" s="3" t="n"/>
+      <c r="C89" s="3" t="n"/>
+      <c r="D89" s="3" t="n"/>
+      <c r="E89" s="3" t="n"/>
       <c r="F89" s="3" t="n"/>
-      <c r="G89" s="3" t="inlineStr"/>
-      <c r="H89" s="3" t="inlineStr"/>
+      <c r="G89" s="3" t="n"/>
+      <c r="H89" s="3" t="n"/>
     </row>
     <row r="90">
-      <c r="A90" s="3" t="n"/>
+      <c r="A90" s="2" t="inlineStr">
+        <is>
+          <t>SECTION 14 — PREPAID EXPENSES</t>
+        </is>
+      </c>
       <c r="B90" s="3" t="n"/>
       <c r="C90" s="3" t="n"/>
       <c r="D90" s="3" t="n"/>
@@ -2829,15 +2899,31 @@
       <c r="H90" s="3" t="n"/>
     </row>
     <row r="91">
-      <c r="A91" s="2" t="inlineStr">
-        <is>
-          <t>SECTION 21 — ACCRUED PAYROLL &amp; RELATED EXPENSES</t>
-        </is>
-      </c>
-      <c r="B91" s="3" t="n"/>
-      <c r="C91" s="3" t="n"/>
-      <c r="D91" s="3" t="n"/>
-      <c r="E91" s="3" t="n"/>
+      <c r="A91" s="3" t="inlineStr">
+        <is>
+          <t>1400</t>
+        </is>
+      </c>
+      <c r="B91" s="3" t="inlineStr">
+        <is>
+          <t>Prepaid Expenses Leadsheet</t>
+        </is>
+      </c>
+      <c r="C91" s="3" t="inlineStr">
+        <is>
+          <t>Workpaper</t>
+        </is>
+      </c>
+      <c r="D91" s="3" t="inlineStr">
+        <is>
+          <t>Leadsheet — prepaids</t>
+        </is>
+      </c>
+      <c r="E91" s="3" t="inlineStr">
+        <is>
+          <t>0900</t>
+        </is>
+      </c>
       <c r="F91" s="3" t="n"/>
       <c r="G91" s="3" t="n"/>
       <c r="H91" s="3" t="n"/>
@@ -2845,69 +2931,53 @@
     <row r="92">
       <c r="A92" s="3" t="inlineStr">
         <is>
-          <t>2100</t>
+          <t>1400-PROG</t>
         </is>
       </c>
       <c r="B92" s="3" t="inlineStr">
         <is>
-          <t>Accrued Expenses Leadsheet</t>
+          <t>AUD-807 Audit Program Ppds, Dfrds, Coll Items, Oth Assets</t>
         </is>
       </c>
       <c r="C92" s="3" t="inlineStr">
         <is>
-          <t>Workpaper</t>
+          <t>KC Form</t>
         </is>
       </c>
       <c r="D92" s="3" t="inlineStr">
         <is>
-          <t>Leadsheet — accrued expenses</t>
+          <t>Audit program — prepaids</t>
         </is>
       </c>
       <c r="E92" s="3" t="inlineStr">
         <is>
-          <t>0900</t>
+          <t>0203, 0500</t>
         </is>
       </c>
       <c r="F92" s="3" t="n"/>
       <c r="G92" s="3" t="n"/>
-      <c r="H92" s="3" t="n"/>
+      <c r="H92" s="3" t="inlineStr">
+        <is>
+          <t>AUD-806</t>
+        </is>
+      </c>
     </row>
     <row r="93">
-      <c r="A93" s="3" t="inlineStr">
-        <is>
-          <t>2100-PROG</t>
-        </is>
-      </c>
-      <c r="B93" s="3" t="inlineStr">
-        <is>
-          <t>AUD-811 Audit Program Payroll and Related Liabilities</t>
-        </is>
-      </c>
-      <c r="C93" s="3" t="inlineStr">
-        <is>
-          <t>KC Form</t>
-        </is>
-      </c>
-      <c r="D93" s="3" t="inlineStr">
-        <is>
-          <t>Audit program — payroll/accrued expenses</t>
-        </is>
-      </c>
-      <c r="E93" s="3" t="inlineStr">
-        <is>
-          <t>0203, 0500</t>
-        </is>
-      </c>
+      <c r="A93" s="3" t="n"/>
+      <c r="B93" s="3" t="n"/>
+      <c r="C93" s="3" t="n"/>
+      <c r="D93" s="3" t="n"/>
+      <c r="E93" s="3" t="n"/>
       <c r="F93" s="3" t="n"/>
       <c r="G93" s="3" t="n"/>
-      <c r="H93" s="3" t="inlineStr">
-        <is>
-          <t>AUD-809</t>
-        </is>
-      </c>
+      <c r="H93" s="3" t="n"/>
     </row>
     <row r="94">
-      <c r="A94" s="3" t="n"/>
+      <c r="A94" s="2" t="inlineStr">
+        <is>
+          <t>SECTION 15 — PROPERTY &amp; EQUIPMENT</t>
+        </is>
+      </c>
       <c r="B94" s="3" t="n"/>
       <c r="C94" s="3" t="n"/>
       <c r="D94" s="3" t="n"/>
@@ -2917,142 +2987,173 @@
       <c r="H94" s="3" t="n"/>
     </row>
     <row r="95">
-      <c r="A95" s="2" t="inlineStr">
-        <is>
-          <t>SECTION 22 — DEFERRED REVENUE</t>
-        </is>
-      </c>
-      <c r="B95" s="3" t="n"/>
-      <c r="C95" s="3" t="n"/>
-      <c r="D95" s="3" t="n"/>
-      <c r="E95" s="3" t="n"/>
-      <c r="F95" s="3" t="n"/>
-      <c r="G95" s="3" t="n"/>
+      <c r="A95" s="3" t="inlineStr">
+        <is>
+          <t>1500</t>
+        </is>
+      </c>
+      <c r="B95" s="3" t="inlineStr">
+        <is>
+          <t>Property &amp; Equipment Leadsheet</t>
+        </is>
+      </c>
+      <c r="C95" s="3" t="inlineStr">
+        <is>
+          <t>Workpaper</t>
+        </is>
+      </c>
+      <c r="D95" s="3" t="inlineStr">
+        <is>
+          <t>Leadsheet — PP&amp;E and depreciation</t>
+        </is>
+      </c>
+      <c r="E95" s="3" t="inlineStr">
+        <is>
+          <t>0900</t>
+        </is>
+      </c>
+      <c r="F95" s="3" t="inlineStr">
+        <is>
+          <t>Add when TB carries property &amp; equipment</t>
+        </is>
+      </c>
+      <c r="G95" s="3" t="inlineStr">
+        <is>
+          <t>if-ppe</t>
+        </is>
+      </c>
       <c r="H95" s="3" t="n"/>
     </row>
     <row r="96">
       <c r="A96" s="3" t="inlineStr">
         <is>
-          <t>2200</t>
+          <t>1500-PROG</t>
         </is>
       </c>
       <c r="B96" s="3" t="inlineStr">
         <is>
-          <t>Deferred Revenue Leadsheet</t>
+          <t>AUD-809 Audit Program Ppty and Equip, and Depr Incl Cntrib Ppty</t>
         </is>
       </c>
       <c r="C96" s="3" t="inlineStr">
         <is>
+          <t>KC Form</t>
+        </is>
+      </c>
+      <c r="D96" s="3" t="inlineStr">
+        <is>
+          <t>Audit program — property &amp; equipment, depreciation, contributed property</t>
+        </is>
+      </c>
+      <c r="E96" s="3" t="inlineStr">
+        <is>
+          <t>0203, 0500</t>
+        </is>
+      </c>
+      <c r="F96" s="3" t="inlineStr">
+        <is>
+          <t>TB-driven — add when TB carries PP&amp;E (KBA-400 scoping confirms)</t>
+        </is>
+      </c>
+      <c r="G96" s="3" t="inlineStr">
+        <is>
+          <t>if-ppe</t>
+        </is>
+      </c>
+      <c r="H96" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="97"/>
+    <row r="98">
+      <c r="A98" s="2" t="inlineStr">
+        <is>
+          <t>SECTION 20 — PAYABLES</t>
+        </is>
+      </c>
+      <c r="B98" s="3" t="n"/>
+      <c r="C98" s="3" t="n"/>
+      <c r="D98" s="3" t="n"/>
+      <c r="E98" s="3" t="n"/>
+      <c r="F98" s="3" t="n"/>
+      <c r="G98" s="3" t="n"/>
+      <c r="H98" s="3" t="n"/>
+    </row>
+    <row r="99">
+      <c r="A99" s="3" t="inlineStr">
+        <is>
+          <t>2000</t>
+        </is>
+      </c>
+      <c r="B99" s="3" t="inlineStr">
+        <is>
+          <t>Payables Leadsheet</t>
+        </is>
+      </c>
+      <c r="C99" s="3" t="inlineStr">
+        <is>
           <t>Workpaper</t>
         </is>
       </c>
-      <c r="D96" s="3" t="inlineStr">
-        <is>
-          <t>Leadsheet — deferred revenue</t>
-        </is>
-      </c>
-      <c r="E96" s="3" t="inlineStr">
+      <c r="D99" s="3" t="inlineStr">
+        <is>
+          <t>Leadsheet — payables</t>
+        </is>
+      </c>
+      <c r="E99" s="3" t="inlineStr">
         <is>
           <t>0900</t>
         </is>
       </c>
-      <c r="F96" s="3" t="n"/>
-      <c r="G96" s="3" t="inlineStr"/>
-      <c r="H96" s="3" t="inlineStr"/>
-    </row>
-    <row r="97">
-      <c r="A97" s="3" t="inlineStr">
-        <is>
-          <t>2201</t>
-        </is>
-      </c>
-      <c r="B97" s="3" t="inlineStr">
-        <is>
-          <t>FY25 NIN SEFA Rollforward</t>
-        </is>
-      </c>
-      <c r="C97" s="3" t="inlineStr">
-        <is>
-          <t>Workpaper</t>
-        </is>
-      </c>
-      <c r="D97" s="3" t="inlineStr">
-        <is>
-          <t>SEFA rollforward schedule</t>
-        </is>
-      </c>
-      <c r="E97" s="3" t="inlineStr">
-        <is>
-          <t>Client</t>
-        </is>
-      </c>
-      <c r="F97" s="3" t="n"/>
-      <c r="G97" s="3" t="inlineStr"/>
-      <c r="H97" s="3" t="inlineStr"/>
-    </row>
-    <row r="98">
-      <c r="A98" s="3" t="inlineStr">
-        <is>
-          <t>2202</t>
-        </is>
-      </c>
-      <c r="B98" s="3" t="inlineStr">
-        <is>
-          <t>Cash Receipts</t>
-        </is>
-      </c>
-      <c r="C98" s="3" t="inlineStr">
-        <is>
-          <t>Workpaper</t>
-        </is>
-      </c>
-      <c r="D98" s="3" t="inlineStr">
-        <is>
-          <t>Cash receipts detail supporting deferred revenue</t>
-        </is>
-      </c>
-      <c r="E98" s="3" t="inlineStr">
-        <is>
-          <t>Client</t>
-        </is>
-      </c>
-      <c r="F98" s="3" t="n"/>
-      <c r="G98" s="3" t="inlineStr"/>
-      <c r="H98" s="3" t="inlineStr"/>
-    </row>
-    <row r="99">
-      <c r="A99" s="3" t="n"/>
-      <c r="B99" s="3" t="n"/>
-      <c r="C99" s="3" t="n"/>
-      <c r="D99" s="3" t="n"/>
-      <c r="E99" s="3" t="n"/>
       <c r="F99" s="3" t="n"/>
       <c r="G99" s="3" t="n"/>
       <c r="H99" s="3" t="n"/>
     </row>
     <row r="100">
-      <c r="A100" s="2" t="inlineStr">
-        <is>
-          <t>SECTION 29 — INTERFUND / DUE TO-FROM AFFILIATES</t>
-        </is>
-      </c>
-      <c r="B100" s="3" t="n"/>
-      <c r="C100" s="3" t="n"/>
-      <c r="D100" s="3" t="n"/>
-      <c r="E100" s="3" t="n"/>
+      <c r="A100" s="3" t="inlineStr">
+        <is>
+          <t>2000-PROG</t>
+        </is>
+      </c>
+      <c r="B100" s="3" t="inlineStr">
+        <is>
+          <t>AUD-810 Audit Program Accounts Payable and Purchases</t>
+        </is>
+      </c>
+      <c r="C100" s="3" t="inlineStr">
+        <is>
+          <t>KC Form</t>
+        </is>
+      </c>
+      <c r="D100" s="3" t="inlineStr">
+        <is>
+          <t>Audit program — AP</t>
+        </is>
+      </c>
+      <c r="E100" s="3" t="inlineStr">
+        <is>
+          <t>0203, 0500</t>
+        </is>
+      </c>
       <c r="F100" s="3" t="n"/>
       <c r="G100" s="3" t="n"/>
-      <c r="H100" s="3" t="n"/>
+      <c r="H100" s="3" t="inlineStr">
+        <is>
+          <t>AUD-808</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="3" t="inlineStr">
         <is>
-          <t>2900</t>
+          <t>2001</t>
         </is>
       </c>
       <c r="B101" s="3" t="inlineStr">
         <is>
-          <t>Interfund/Due to Affiliates Leadsheet</t>
+          <t>Search for Unrecorded Liabilities</t>
         </is>
       </c>
       <c r="C101" s="3" t="inlineStr">
@@ -3062,12 +3163,12 @@
       </c>
       <c r="D101" s="3" t="inlineStr">
         <is>
-          <t>Leadsheet — interfund balances</t>
+          <t>SUL testing workpaper</t>
         </is>
       </c>
       <c r="E101" s="3" t="inlineStr">
         <is>
-          <t>0900</t>
+          <t>2000-PROG</t>
         </is>
       </c>
       <c r="F101" s="3" t="n"/>
@@ -3087,7 +3188,7 @@
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
         <is>
-          <t>SECTION 30 — NET ASSETS</t>
+          <t>SECTION 21 — ACCRUED PAYROLL &amp; RELATED EXPENSES</t>
         </is>
       </c>
       <c r="B103" s="3" t="n"/>
@@ -3101,12 +3202,12 @@
     <row r="104">
       <c r="A104" s="3" t="inlineStr">
         <is>
-          <t>3000</t>
+          <t>2100</t>
         </is>
       </c>
       <c r="B104" s="3" t="inlineStr">
         <is>
-          <t>Equity Leadsheet</t>
+          <t>Accrued Expenses Leadsheet</t>
         </is>
       </c>
       <c r="C104" s="3" t="inlineStr">
@@ -3116,7 +3217,7 @@
       </c>
       <c r="D104" s="3" t="inlineStr">
         <is>
-          <t>Leadsheet — equity/net position</t>
+          <t>Leadsheet — accrued expenses</t>
         </is>
       </c>
       <c r="E104" s="3" t="inlineStr">
@@ -3131,12 +3232,12 @@
     <row r="105">
       <c r="A105" s="3" t="inlineStr">
         <is>
-          <t>3000-PROG</t>
+          <t>2100-PROG</t>
         </is>
       </c>
       <c r="B105" s="3" t="inlineStr">
         <is>
-          <t>AUD-814 Audit Program Net Assets</t>
+          <t>AUD-811 Audit Program Payroll and Related Liabilities</t>
         </is>
       </c>
       <c r="C105" s="3" t="inlineStr">
@@ -3146,7 +3247,7 @@
       </c>
       <c r="D105" s="3" t="inlineStr">
         <is>
-          <t>Audit program — equity/fund balance</t>
+          <t>Audit program — payroll/accrued expenses</t>
         </is>
       </c>
       <c r="E105" s="3" t="inlineStr">
@@ -3158,7 +3259,7 @@
       <c r="G105" s="3" t="n"/>
       <c r="H105" s="3" t="inlineStr">
         <is>
-          <t>AUD-811</t>
+          <t>AUD-809</t>
         </is>
       </c>
     </row>
@@ -3175,7 +3276,7 @@
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
         <is>
-          <t>SECTION 40 — REVENUES</t>
+          <t>SECTION 22 — DEFERRED REVENUE</t>
         </is>
       </c>
       <c r="B107" s="3" t="n"/>
@@ -3189,12 +3290,12 @@
     <row r="108">
       <c r="A108" s="3" t="inlineStr">
         <is>
-          <t>4000</t>
+          <t>2200</t>
         </is>
       </c>
       <c r="B108" s="3" t="inlineStr">
         <is>
-          <t>Revenue Leadsheet</t>
+          <t>Deferred Revenue Leadsheet</t>
         </is>
       </c>
       <c r="C108" s="3" t="inlineStr">
@@ -3204,7 +3305,7 @@
       </c>
       <c r="D108" s="3" t="inlineStr">
         <is>
-          <t>Leadsheet — revenues</t>
+          <t>Leadsheet — deferred revenue</t>
         </is>
       </c>
       <c r="E108" s="3" t="inlineStr">
@@ -3219,12 +3320,12 @@
     <row r="109">
       <c r="A109" s="3" t="inlineStr">
         <is>
-          <t>4001</t>
+          <t>2201</t>
         </is>
       </c>
       <c r="B109" s="3" t="inlineStr">
         <is>
-          <t>Other Operating Revenue Leadsheet</t>
+          <t>FY25 NIN SEFA Rollforward</t>
         </is>
       </c>
       <c r="C109" s="3" t="inlineStr">
@@ -3234,12 +3335,12 @@
       </c>
       <c r="D109" s="3" t="inlineStr">
         <is>
-          <t>Leadsheet — other operating revenue</t>
+          <t>SEFA rollforward schedule</t>
         </is>
       </c>
       <c r="E109" s="3" t="inlineStr">
         <is>
-          <t>0900</t>
+          <t>Client</t>
         </is>
       </c>
       <c r="F109" s="3" t="n"/>
@@ -3247,21 +3348,37 @@
       <c r="H109" s="3" t="inlineStr"/>
     </row>
     <row r="110">
-      <c r="A110" s="3" t="n"/>
-      <c r="B110" s="3" t="n"/>
-      <c r="C110" s="3" t="n"/>
-      <c r="D110" s="3" t="n"/>
-      <c r="E110" s="3" t="n"/>
+      <c r="A110" s="3" t="inlineStr">
+        <is>
+          <t>2202</t>
+        </is>
+      </c>
+      <c r="B110" s="3" t="inlineStr">
+        <is>
+          <t>Cash Receipts</t>
+        </is>
+      </c>
+      <c r="C110" s="3" t="inlineStr">
+        <is>
+          <t>Workpaper</t>
+        </is>
+      </c>
+      <c r="D110" s="3" t="inlineStr">
+        <is>
+          <t>Cash receipts detail supporting deferred revenue</t>
+        </is>
+      </c>
+      <c r="E110" s="3" t="inlineStr">
+        <is>
+          <t>Client</t>
+        </is>
+      </c>
       <c r="F110" s="3" t="n"/>
-      <c r="G110" s="3" t="n"/>
-      <c r="H110" s="3" t="n"/>
+      <c r="G110" s="3" t="inlineStr"/>
+      <c r="H110" s="3" t="inlineStr"/>
     </row>
     <row r="111">
-      <c r="A111" s="2" t="inlineStr">
-        <is>
-          <t>SECTION 50 — EXPENSES</t>
-        </is>
-      </c>
+      <c r="A111" s="3" t="n"/>
       <c r="B111" s="3" t="n"/>
       <c r="C111" s="3" t="n"/>
       <c r="D111" s="3" t="n"/>
@@ -3271,51 +3388,51 @@
       <c r="H111" s="3" t="n"/>
     </row>
     <row r="112">
-      <c r="A112" s="3" t="inlineStr">
-        <is>
-          <t>5000</t>
-        </is>
-      </c>
-      <c r="B112" s="3" t="inlineStr">
-        <is>
-          <t>Expenses Leadsheet</t>
-        </is>
-      </c>
-      <c r="C112" s="3" t="inlineStr">
+      <c r="A112" s="2" t="inlineStr">
+        <is>
+          <t>SECTION 29 — INTERFUND / DUE TO-FROM AFFILIATES</t>
+        </is>
+      </c>
+      <c r="B112" s="3" t="n"/>
+      <c r="C112" s="3" t="n"/>
+      <c r="D112" s="3" t="n"/>
+      <c r="E112" s="3" t="n"/>
+      <c r="F112" s="3" t="n"/>
+      <c r="G112" s="3" t="n"/>
+      <c r="H112" s="3" t="n"/>
+    </row>
+    <row r="113">
+      <c r="A113" s="3" t="inlineStr">
+        <is>
+          <t>2900</t>
+        </is>
+      </c>
+      <c r="B113" s="3" t="inlineStr">
+        <is>
+          <t>Interfund/Due to Affiliates Leadsheet</t>
+        </is>
+      </c>
+      <c r="C113" s="3" t="inlineStr">
         <is>
           <t>Workpaper</t>
         </is>
       </c>
-      <c r="D112" s="3" t="inlineStr">
-        <is>
-          <t>Leadsheet — expenses</t>
-        </is>
-      </c>
-      <c r="E112" s="3" t="inlineStr">
+      <c r="D113" s="3" t="inlineStr">
+        <is>
+          <t>Leadsheet — interfund balances</t>
+        </is>
+      </c>
+      <c r="E113" s="3" t="inlineStr">
         <is>
           <t>0900</t>
         </is>
       </c>
-      <c r="F112" s="3" t="n"/>
-      <c r="G112" s="3" t="inlineStr"/>
-      <c r="H112" s="3" t="inlineStr"/>
-    </row>
-    <row r="113">
-      <c r="A113" s="3" t="n"/>
-      <c r="B113" s="3" t="n"/>
-      <c r="C113" s="3" t="n"/>
-      <c r="D113" s="3" t="n"/>
-      <c r="E113" s="3" t="n"/>
       <c r="F113" s="3" t="n"/>
-      <c r="G113" s="3" t="n"/>
-      <c r="H113" s="3" t="n"/>
+      <c r="G113" s="3" t="inlineStr"/>
+      <c r="H113" s="3" t="inlineStr"/>
     </row>
     <row r="114">
-      <c r="A114" s="2" t="inlineStr">
-        <is>
-          <t>SECTION 70 — TRANSFERS</t>
-        </is>
-      </c>
+      <c r="A114" s="3" t="n"/>
       <c r="B114" s="3" t="n"/>
       <c r="C114" s="3" t="n"/>
       <c r="D114" s="3" t="n"/>
@@ -3325,186 +3442,146 @@
       <c r="H114" s="3" t="n"/>
     </row>
     <row r="115">
-      <c r="A115" s="3" t="inlineStr">
-        <is>
-          <t>7000</t>
-        </is>
-      </c>
-      <c r="B115" s="3" t="inlineStr">
-        <is>
-          <t>Transfers Leadsheet</t>
-        </is>
-      </c>
-      <c r="C115" s="3" t="inlineStr">
+      <c r="A115" s="2" t="inlineStr">
+        <is>
+          <t>SECTION 30 — NET ASSETS</t>
+        </is>
+      </c>
+      <c r="B115" s="3" t="n"/>
+      <c r="C115" s="3" t="n"/>
+      <c r="D115" s="3" t="n"/>
+      <c r="E115" s="3" t="n"/>
+      <c r="F115" s="3" t="n"/>
+      <c r="G115" s="3" t="n"/>
+      <c r="H115" s="3" t="n"/>
+    </row>
+    <row r="116">
+      <c r="A116" s="3" t="inlineStr">
+        <is>
+          <t>3000</t>
+        </is>
+      </c>
+      <c r="B116" s="3" t="inlineStr">
+        <is>
+          <t>Equity Leadsheet</t>
+        </is>
+      </c>
+      <c r="C116" s="3" t="inlineStr">
         <is>
           <t>Workpaper</t>
         </is>
       </c>
-      <c r="D115" s="3" t="inlineStr">
-        <is>
-          <t>Leadsheet — transfers</t>
-        </is>
-      </c>
-      <c r="E115" s="3" t="inlineStr">
+      <c r="D116" s="3" t="inlineStr">
+        <is>
+          <t>Leadsheet — equity/net position</t>
+        </is>
+      </c>
+      <c r="E116" s="3" t="inlineStr">
         <is>
           <t>0900</t>
         </is>
       </c>
-      <c r="F115" s="3" t="n"/>
-      <c r="G115" s="3" t="inlineStr"/>
-      <c r="H115" s="3" t="inlineStr"/>
-    </row>
-    <row r="116">
-      <c r="A116" s="3" t="n"/>
-      <c r="B116" s="3" t="n"/>
-      <c r="C116" s="3" t="n"/>
-      <c r="D116" s="3" t="n"/>
-      <c r="E116" s="3" t="n"/>
       <c r="F116" s="3" t="n"/>
       <c r="G116" s="3" t="n"/>
       <c r="H116" s="3" t="n"/>
     </row>
     <row r="117">
-      <c r="A117" s="2" t="inlineStr">
-        <is>
-          <t>SECTION 80 — SINGLE AUDIT: PLANNING</t>
-        </is>
-      </c>
-      <c r="B117" s="3" t="n"/>
-      <c r="C117" s="3" t="n"/>
-      <c r="D117" s="3" t="n"/>
-      <c r="E117" s="3" t="n"/>
+      <c r="A117" s="3" t="inlineStr">
+        <is>
+          <t>3000-PROG</t>
+        </is>
+      </c>
+      <c r="B117" s="3" t="inlineStr">
+        <is>
+          <t>AUD-814 Audit Program Net Assets</t>
+        </is>
+      </c>
+      <c r="C117" s="3" t="inlineStr">
+        <is>
+          <t>KC Form</t>
+        </is>
+      </c>
+      <c r="D117" s="3" t="inlineStr">
+        <is>
+          <t>Audit program — equity/fund balance</t>
+        </is>
+      </c>
+      <c r="E117" s="3" t="inlineStr">
+        <is>
+          <t>0203, 0500</t>
+        </is>
+      </c>
       <c r="F117" s="3" t="n"/>
       <c r="G117" s="3" t="n"/>
-      <c r="H117" s="3" t="n"/>
+      <c r="H117" s="3" t="inlineStr">
+        <is>
+          <t>AUD-811</t>
+        </is>
+      </c>
     </row>
     <row r="118">
-      <c r="A118" s="3" t="inlineStr">
-        <is>
-          <t>8000</t>
-        </is>
-      </c>
-      <c r="B118" s="3" t="inlineStr">
-        <is>
-          <t>AUD-100S Engagement-Level Tailoring Questions — Uniform Guidance</t>
-        </is>
-      </c>
-      <c r="C118" s="3" t="inlineStr">
-        <is>
-          <t>KC Form</t>
-        </is>
-      </c>
-      <c r="D118" s="3" t="inlineStr">
-        <is>
-          <t>SA tailoring; drives SA-specific KC form content — complete before other 8000s</t>
-        </is>
-      </c>
-      <c r="E118" s="3" t="inlineStr">
-        <is>
-          <t>0101</t>
-        </is>
-      </c>
-      <c r="F118" s="3" t="inlineStr">
-        <is>
-          <t>Complete before other 8000-series KC forms</t>
-        </is>
-      </c>
-      <c r="G118" s="3" t="inlineStr">
-        <is>
-          <t>if-single-audit</t>
-        </is>
-      </c>
-      <c r="H118" s="3" t="inlineStr">
-        <is>
-          <t>AUD-100S</t>
-        </is>
-      </c>
+      <c r="A118" s="3" t="n"/>
+      <c r="B118" s="3" t="n"/>
+      <c r="C118" s="3" t="n"/>
+      <c r="D118" s="3" t="n"/>
+      <c r="E118" s="3" t="n"/>
+      <c r="F118" s="3" t="n"/>
+      <c r="G118" s="3" t="n"/>
+      <c r="H118" s="3" t="n"/>
     </row>
     <row r="119">
-      <c r="A119" s="3" t="inlineStr">
-        <is>
-          <t>8000.1</t>
-        </is>
-      </c>
-      <c r="B119" s="3" t="inlineStr">
-        <is>
-          <t>AUD-101S Overall Audit Program — Uniform Guidance</t>
-        </is>
-      </c>
-      <c r="C119" s="3" t="inlineStr">
-        <is>
-          <t>KC Form</t>
-        </is>
-      </c>
-      <c r="D119" s="3" t="inlineStr">
-        <is>
-          <t>SA master audit program roadmap</t>
-        </is>
-      </c>
-      <c r="E119" s="3" t="inlineStr">
-        <is>
-          <t>8000</t>
-        </is>
-      </c>
+      <c r="A119" s="2" t="inlineStr">
+        <is>
+          <t>SECTION 40 — REVENUES</t>
+        </is>
+      </c>
+      <c r="B119" s="3" t="n"/>
+      <c r="C119" s="3" t="n"/>
+      <c r="D119" s="3" t="n"/>
+      <c r="E119" s="3" t="n"/>
       <c r="F119" s="3" t="n"/>
-      <c r="G119" s="3" t="inlineStr">
-        <is>
-          <t>if-single-audit</t>
-        </is>
-      </c>
-      <c r="H119" s="3" t="inlineStr">
-        <is>
-          <t>AUD-101S</t>
-        </is>
-      </c>
+      <c r="G119" s="3" t="n"/>
+      <c r="H119" s="3" t="n"/>
     </row>
     <row r="120">
       <c r="A120" s="3" t="inlineStr">
         <is>
-          <t>8001</t>
+          <t>4000</t>
         </is>
       </c>
       <c r="B120" s="3" t="inlineStr">
         <is>
-          <t>KBA-101S Overall Uniform Guidance Compliance Audit Strategy</t>
+          <t>Revenue Leadsheet</t>
         </is>
       </c>
       <c r="C120" s="3" t="inlineStr">
         <is>
-          <t>KC Form</t>
+          <t>Workpaper</t>
         </is>
       </c>
       <c r="D120" s="3" t="inlineStr">
         <is>
-          <t>SA audit strategy</t>
+          <t>Leadsheet — revenues</t>
         </is>
       </c>
       <c r="E120" s="3" t="inlineStr">
         <is>
-          <t>8000, 8000.1</t>
+          <t>0900</t>
         </is>
       </c>
       <c r="F120" s="3" t="n"/>
-      <c r="G120" s="3" t="inlineStr">
-        <is>
-          <t>if-single-audit</t>
-        </is>
-      </c>
-      <c r="H120" s="3" t="inlineStr">
-        <is>
-          <t>KBA-101S</t>
-        </is>
-      </c>
+      <c r="G120" s="3" t="inlineStr"/>
+      <c r="H120" s="3" t="inlineStr"/>
     </row>
     <row r="121">
       <c r="A121" s="3" t="inlineStr">
         <is>
-          <t>8001.1</t>
+          <t>4000-PROG</t>
         </is>
       </c>
       <c r="B121" s="3" t="inlineStr">
         <is>
-          <t>KBA-302S Understanding Entity and Its Program Environment</t>
+          <t>AUD-805 Audit Program Cntrib Rec, Supp, Progr Rev and Agcy Tran</t>
         </is>
       </c>
       <c r="C121" s="3" t="inlineStr">
@@ -3514,309 +3591,185 @@
       </c>
       <c r="D121" s="3" t="inlineStr">
         <is>
-          <t>Entity program environment understanding</t>
+          <t>Audit program — contributions receivable, support, program revenue, agency transactions</t>
         </is>
       </c>
       <c r="E121" s="3" t="inlineStr">
         <is>
-          <t>8001, 0300</t>
-        </is>
-      </c>
-      <c r="F121" s="3" t="n"/>
+          <t>0203, 0500</t>
+        </is>
+      </c>
+      <c r="F121" s="3" t="inlineStr">
+        <is>
+          <t>TB-driven — add when TB carries contributions/support revenue (most NPOs; KBA-400 scoping confirms)</t>
+        </is>
+      </c>
       <c r="G121" s="3" t="inlineStr">
         <is>
-          <t>if-single-audit</t>
+          <t>if-contributions</t>
         </is>
       </c>
       <c r="H121" s="3" t="inlineStr">
         <is>
-          <t>KBA-302S</t>
+          <t>—</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" s="3" t="inlineStr">
         <is>
-          <t>8001.2</t>
+          <t>4001</t>
         </is>
       </c>
       <c r="B122" s="3" t="inlineStr">
         <is>
-          <t>KBA-503S Basis for Assessment of Inherent Risk of Noncompliance</t>
+          <t>Other Operating Revenue Leadsheet</t>
         </is>
       </c>
       <c r="C122" s="3" t="inlineStr">
         <is>
-          <t>KC Form</t>
+          <t>Workpaper</t>
         </is>
       </c>
       <c r="D122" s="3" t="inlineStr">
         <is>
-          <t>IR assessment for compliance</t>
+          <t>Leadsheet — other operating revenue</t>
         </is>
       </c>
       <c r="E122" s="3" t="inlineStr">
         <is>
-          <t>8001.1, 0501</t>
+          <t>0900</t>
         </is>
       </c>
       <c r="F122" s="3" t="n"/>
-      <c r="G122" s="3" t="inlineStr">
-        <is>
-          <t>if-single-audit</t>
-        </is>
-      </c>
-      <c r="H122" s="3" t="inlineStr">
-        <is>
-          <t>KBA-503S</t>
-        </is>
-      </c>
+      <c r="G122" s="3" t="inlineStr"/>
+      <c r="H122" s="3" t="inlineStr"/>
     </row>
     <row r="123">
-      <c r="A123" s="3" t="inlineStr">
-        <is>
-          <t>8002</t>
-        </is>
-      </c>
-      <c r="B123" s="3" t="inlineStr">
-        <is>
-          <t>KBA-301S Compliance Requirement Materiality</t>
-        </is>
-      </c>
-      <c r="C123" s="3" t="inlineStr">
-        <is>
-          <t>KC Form</t>
-        </is>
-      </c>
-      <c r="D123" s="3" t="inlineStr">
-        <is>
-          <t>Materiality at major program and compliance requirement levels</t>
-        </is>
-      </c>
-      <c r="E123" s="3" t="inlineStr">
-        <is>
-          <t>0202, 8001</t>
-        </is>
-      </c>
+      <c r="A123" s="3" t="n"/>
+      <c r="B123" s="3" t="n"/>
+      <c r="C123" s="3" t="n"/>
+      <c r="D123" s="3" t="n"/>
+      <c r="E123" s="3" t="n"/>
       <c r="F123" s="3" t="n"/>
-      <c r="G123" s="3" t="inlineStr">
-        <is>
-          <t>if-single-audit</t>
-        </is>
-      </c>
-      <c r="H123" s="3" t="inlineStr">
-        <is>
-          <t>KBA-301S</t>
-        </is>
-      </c>
+      <c r="G123" s="3" t="n"/>
+      <c r="H123" s="3" t="n"/>
     </row>
     <row r="124">
-      <c r="A124" s="3" t="inlineStr">
-        <is>
-          <t>8003</t>
-        </is>
-      </c>
-      <c r="B124" s="3" t="inlineStr">
-        <is>
-          <t>AID-301S Audit Applicability and Major Programs (SA-18)</t>
-        </is>
-      </c>
-      <c r="C124" s="3" t="inlineStr">
-        <is>
-          <t>KC Form</t>
-        </is>
-      </c>
-      <c r="D124" s="3" t="inlineStr">
-        <is>
-          <t>Major program determination — drives which 8100+ sections exist</t>
-        </is>
-      </c>
-      <c r="E124" s="3" t="inlineStr">
-        <is>
-          <t>2201 (SEFA), 8002</t>
-        </is>
-      </c>
-      <c r="F124" s="3" t="inlineStr">
-        <is>
-          <t>Complete before KBA-502S; drives risk scope</t>
-        </is>
-      </c>
-      <c r="G124" s="3" t="inlineStr">
-        <is>
-          <t>if-single-audit</t>
-        </is>
-      </c>
-      <c r="H124" s="3" t="inlineStr">
-        <is>
-          <t>AID-301S</t>
-        </is>
-      </c>
+      <c r="A124" s="2" t="inlineStr">
+        <is>
+          <t>SECTION 50 — EXPENSES</t>
+        </is>
+      </c>
+      <c r="B124" s="3" t="n"/>
+      <c r="C124" s="3" t="n"/>
+      <c r="D124" s="3" t="n"/>
+      <c r="E124" s="3" t="n"/>
+      <c r="F124" s="3" t="n"/>
+      <c r="G124" s="3" t="n"/>
+      <c r="H124" s="3" t="n"/>
     </row>
     <row r="125">
       <c r="A125" s="3" t="inlineStr">
         <is>
-          <t>8004</t>
+          <t>5000</t>
         </is>
       </c>
       <c r="B125" s="3" t="inlineStr">
         <is>
-          <t>KBA-502S Summary of Risk Assessments — Noncompliance</t>
+          <t>Expenses Leadsheet</t>
         </is>
       </c>
       <c r="C125" s="3" t="inlineStr">
         <is>
-          <t>KC Form</t>
+          <t>Workpaper</t>
         </is>
       </c>
       <c r="D125" s="3" t="inlineStr">
         <is>
-          <t>Compliance risk summary by requirement; living document</t>
+          <t>Leadsheet — expenses</t>
         </is>
       </c>
       <c r="E125" s="3" t="inlineStr">
         <is>
-          <t>8003, 8001.2</t>
+          <t>0900</t>
         </is>
       </c>
       <c r="F125" s="3" t="n"/>
-      <c r="G125" s="3" t="inlineStr">
-        <is>
-          <t>if-single-audit</t>
-        </is>
-      </c>
-      <c r="H125" s="3" t="inlineStr">
-        <is>
-          <t>KBA-502S</t>
-        </is>
-      </c>
+      <c r="G125" s="3" t="inlineStr"/>
+      <c r="H125" s="3" t="inlineStr"/>
     </row>
     <row r="126">
-      <c r="A126" s="3" t="inlineStr">
-        <is>
-          <t>8005</t>
-        </is>
-      </c>
-      <c r="B126" s="3" t="inlineStr">
-        <is>
-          <t>KBA-102S Uniform Guidance Compliance Audit Significant Matters</t>
-        </is>
-      </c>
-      <c r="C126" s="3" t="inlineStr">
-        <is>
-          <t>KC Form</t>
-        </is>
-      </c>
-      <c r="D126" s="3" t="inlineStr">
-        <is>
-          <t>SA significant matters/completion document</t>
-        </is>
-      </c>
-      <c r="E126" s="3" t="inlineStr">
-        <is>
-          <t>All 8100+ complete</t>
-        </is>
-      </c>
+      <c r="A126" s="3" t="n"/>
+      <c r="B126" s="3" t="n"/>
+      <c r="C126" s="3" t="n"/>
+      <c r="D126" s="3" t="n"/>
+      <c r="E126" s="3" t="n"/>
       <c r="F126" s="3" t="n"/>
-      <c r="G126" s="3" t="inlineStr">
-        <is>
-          <t>if-single-audit</t>
-        </is>
-      </c>
-      <c r="H126" s="3" t="inlineStr">
-        <is>
-          <t>KBA-102S</t>
-        </is>
-      </c>
+      <c r="G126" s="3" t="n"/>
+      <c r="H126" s="3" t="n"/>
     </row>
     <row r="127">
-      <c r="A127" s="3" t="inlineStr">
-        <is>
-          <t>8006</t>
-        </is>
-      </c>
-      <c r="B127" s="3" t="inlineStr">
-        <is>
-          <t>KCO-001 Single Audit Title Overview</t>
-        </is>
-      </c>
-      <c r="C127" s="3" t="inlineStr">
-        <is>
-          <t>KC Form</t>
-        </is>
-      </c>
-      <c r="D127" s="3" t="inlineStr">
-        <is>
-          <t>Knowledge Coach SA overview reference</t>
-        </is>
-      </c>
-      <c r="E127" s="3" t="inlineStr">
-        <is>
-          <t>8000</t>
-        </is>
-      </c>
+      <c r="A127" s="2" t="inlineStr">
+        <is>
+          <t>SECTION 60 — OTHER INCOME &amp; EXPENSE</t>
+        </is>
+      </c>
+      <c r="B127" s="3" t="n"/>
+      <c r="C127" s="3" t="n"/>
+      <c r="D127" s="3" t="n"/>
+      <c r="E127" s="3" t="n"/>
       <c r="F127" s="3" t="n"/>
-      <c r="G127" s="3" t="inlineStr">
-        <is>
-          <t>if-single-audit</t>
-        </is>
-      </c>
-      <c r="H127" s="3" t="inlineStr">
-        <is>
-          <t>KCO-001</t>
-        </is>
-      </c>
+      <c r="G127" s="3" t="n"/>
+      <c r="H127" s="3" t="n"/>
     </row>
     <row r="128">
       <c r="A128" s="3" t="inlineStr">
         <is>
-          <t>8006.1</t>
+          <t>6000</t>
         </is>
       </c>
       <c r="B128" s="3" t="inlineStr">
         <is>
-          <t>KBA-401S Understanding Entity-Level Controls over Compliance</t>
+          <t>Other Income &amp; Expense Leadsheet</t>
         </is>
       </c>
       <c r="C128" s="3" t="inlineStr">
         <is>
-          <t>KC Form</t>
+          <t>Workpaper</t>
         </is>
       </c>
       <c r="D128" s="3" t="inlineStr">
         <is>
-          <t>Entity-level controls specific to federal compliance</t>
+          <t>Leadsheet — other income/expense</t>
         </is>
       </c>
       <c r="E128" s="3" t="inlineStr">
         <is>
-          <t>0400, 8001.1</t>
+          <t>0900</t>
         </is>
       </c>
       <c r="F128" s="3" t="inlineStr">
         <is>
-          <t>8-page form — separate from FS KBA-401</t>
+          <t>Add when TB carries other income/expense</t>
         </is>
       </c>
       <c r="G128" s="3" t="inlineStr">
         <is>
-          <t>if-single-audit</t>
-        </is>
-      </c>
-      <c r="H128" s="3" t="inlineStr">
-        <is>
-          <t>KBA-401S</t>
-        </is>
-      </c>
+          <t>if-other-income-expense</t>
+        </is>
+      </c>
+      <c r="H128" s="3" t="n"/>
     </row>
     <row r="129">
       <c r="A129" s="3" t="inlineStr">
         <is>
-          <t>8006.2</t>
+          <t>6000-PROG</t>
         </is>
       </c>
       <c r="B129" s="3" t="inlineStr">
         <is>
-          <t>AID-401S Understanding General IT Controls over Compliance</t>
+          <t>AUD-815 Audit Program Other Income and Expenditures/Expenses</t>
         </is>
       </c>
       <c r="C129" s="3" t="inlineStr">
@@ -3826,40 +3779,35 @@
       </c>
       <c r="D129" s="3" t="inlineStr">
         <is>
-          <t>IT controls over compliance programs</t>
+          <t>Audit program — other income and expenditures/expenses</t>
         </is>
       </c>
       <c r="E129" s="3" t="inlineStr">
         <is>
-          <t>0400.1, 8006.1</t>
-        </is>
-      </c>
-      <c r="F129" s="3" t="n"/>
+          <t>0203, 0500</t>
+        </is>
+      </c>
+      <c r="F129" s="3" t="inlineStr">
+        <is>
+          <t>TB-driven — add when TB carries other income/expense (KBA-400 scoping confirms)</t>
+        </is>
+      </c>
       <c r="G129" s="3" t="inlineStr">
         <is>
-          <t>if-single-audit</t>
+          <t>if-other-income-expense</t>
         </is>
       </c>
       <c r="H129" s="3" t="inlineStr">
         <is>
-          <t>AID-401S</t>
-        </is>
-      </c>
-    </row>
-    <row r="130">
-      <c r="A130" s="3" t="n"/>
-      <c r="B130" s="3" t="n"/>
-      <c r="C130" s="3" t="n"/>
-      <c r="D130" s="3" t="n"/>
-      <c r="E130" s="3" t="n"/>
-      <c r="F130" s="3" t="n"/>
-      <c r="G130" s="3" t="n"/>
-      <c r="H130" s="3" t="n"/>
-    </row>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="130"/>
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
         <is>
-          <t>SECTION 81 — SINGLE AUDIT: ARPA (CFDA 21.027)</t>
+          <t>SECTION 70 — TRANSFERS</t>
         </is>
       </c>
       <c r="B131" s="3" t="n"/>
@@ -3873,134 +3821,66 @@
     <row r="132">
       <c r="A132" s="3" t="inlineStr">
         <is>
-          <t>8100</t>
+          <t>7000</t>
         </is>
       </c>
       <c r="B132" s="3" t="inlineStr">
         <is>
-          <t>KBA-400S Identification of D&amp;M Compliance Requirements — ARPA</t>
+          <t>Transfers Leadsheet</t>
         </is>
       </c>
       <c r="C132" s="3" t="inlineStr">
         <is>
-          <t>KC Form</t>
+          <t>Workpaper</t>
         </is>
       </c>
       <c r="D132" s="3" t="inlineStr">
         <is>
-          <t>Identifies direct and material compliance requirements; complete before programs</t>
+          <t>Leadsheet — transfers</t>
         </is>
       </c>
       <c r="E132" s="3" t="inlineStr">
         <is>
-          <t>8003, 8001.1</t>
-        </is>
-      </c>
-      <c r="F132" s="3" t="inlineStr">
-        <is>
-          <t>CRITICAL — complete before 8101+</t>
-        </is>
-      </c>
-      <c r="G132" s="3" t="inlineStr">
-        <is>
-          <t>if-single-audit</t>
-        </is>
-      </c>
-      <c r="H132" s="3" t="inlineStr">
-        <is>
-          <t>KBA-400S</t>
-        </is>
-      </c>
+          <t>0900</t>
+        </is>
+      </c>
+      <c r="F132" s="3" t="n"/>
+      <c r="G132" s="3" t="inlineStr"/>
+      <c r="H132" s="3" t="inlineStr"/>
     </row>
     <row r="133">
-      <c r="A133" s="3" t="inlineStr">
-        <is>
-          <t>8100.1</t>
-        </is>
-      </c>
-      <c r="B133" s="3" t="inlineStr">
-        <is>
-          <t>AID-303S Determining Compliance Audit Materiality (SA-18)</t>
-        </is>
-      </c>
-      <c r="C133" s="3" t="inlineStr">
-        <is>
-          <t>Excel</t>
-        </is>
-      </c>
-      <c r="D133" s="3" t="inlineStr">
-        <is>
-          <t>Compliance audit materiality worksheet for ARPA</t>
-        </is>
-      </c>
-      <c r="E133" s="3" t="inlineStr">
-        <is>
-          <t>8002, 8100</t>
-        </is>
-      </c>
-      <c r="F133" s="3" t="inlineStr">
-        <is>
-          <t>Excel workpaper</t>
-        </is>
-      </c>
-      <c r="G133" s="3" t="inlineStr">
-        <is>
-          <t>if-single-audit</t>
-        </is>
-      </c>
-      <c r="H133" s="3" t="inlineStr">
-        <is>
-          <t>AID-303S</t>
-        </is>
-      </c>
+      <c r="A133" s="3" t="n"/>
+      <c r="B133" s="3" t="n"/>
+      <c r="C133" s="3" t="n"/>
+      <c r="D133" s="3" t="n"/>
+      <c r="E133" s="3" t="n"/>
+      <c r="F133" s="3" t="n"/>
+      <c r="G133" s="3" t="n"/>
+      <c r="H133" s="3" t="n"/>
     </row>
     <row r="134">
-      <c r="A134" s="3" t="inlineStr">
-        <is>
-          <t>8100.2</t>
-        </is>
-      </c>
-      <c r="B134" s="3" t="inlineStr">
-        <is>
-          <t>Compliance Supplement — ARPA 21.027 (Highlighted)</t>
-        </is>
-      </c>
-      <c r="C134" s="3" t="inlineStr">
-        <is>
-          <t>Support Doc</t>
-        </is>
-      </c>
-      <c r="D134" s="3" t="inlineStr">
-        <is>
-          <t>Applicable compliance supplement with requirements highlighted</t>
-        </is>
-      </c>
-      <c r="E134" s="3" t="inlineStr">
-        <is>
-          <t>8100</t>
-        </is>
-      </c>
-      <c r="F134" s="3" t="inlineStr">
-        <is>
-          <t>Highlight applicable requirements before testing</t>
-        </is>
-      </c>
-      <c r="G134" s="3" t="inlineStr">
-        <is>
-          <t>if-single-audit</t>
-        </is>
-      </c>
-      <c r="H134" s="3" t="inlineStr"/>
+      <c r="A134" s="2" t="inlineStr">
+        <is>
+          <t>SECTION 80 — SINGLE AUDIT: PLANNING</t>
+        </is>
+      </c>
+      <c r="B134" s="3" t="n"/>
+      <c r="C134" s="3" t="n"/>
+      <c r="D134" s="3" t="n"/>
+      <c r="E134" s="3" t="n"/>
+      <c r="F134" s="3" t="n"/>
+      <c r="G134" s="3" t="n"/>
+      <c r="H134" s="3" t="n"/>
     </row>
     <row r="135">
       <c r="A135" s="3" t="inlineStr">
         <is>
-          <t>8101</t>
+          <t>8000</t>
         </is>
       </c>
       <c r="B135" s="3" t="inlineStr">
         <is>
-          <t>AUD-701S Audit Program Designing Tests of Controls over Compliance — ARPA</t>
+          <t>AUD-100S Engagement-Level Tailoring Questions — Uniform Guidance</t>
         </is>
       </c>
       <c r="C135" s="3" t="inlineStr">
@@ -4010,15 +3890,19 @@
       </c>
       <c r="D135" s="3" t="inlineStr">
         <is>
-          <t>Lead controls testing program for ARPA compliance</t>
+          <t>SA tailoring; drives SA-specific KC form content — complete before other 8000s</t>
         </is>
       </c>
       <c r="E135" s="3" t="inlineStr">
         <is>
-          <t>8006.1, 8100</t>
-        </is>
-      </c>
-      <c r="F135" s="3" t="n"/>
+          <t>0101</t>
+        </is>
+      </c>
+      <c r="F135" s="3" t="inlineStr">
+        <is>
+          <t>Complete before other 8000-series KC forms</t>
+        </is>
+      </c>
       <c r="G135" s="3" t="inlineStr">
         <is>
           <t>if-single-audit</t>
@@ -4026,19 +3910,19 @@
       </c>
       <c r="H135" s="3" t="inlineStr">
         <is>
-          <t>AUD-701S</t>
+          <t>AUD-100S</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" s="3" t="inlineStr">
         <is>
-          <t>8101.1</t>
+          <t>8000.1</t>
         </is>
       </c>
       <c r="B136" s="3" t="inlineStr">
         <is>
-          <t>AUD-801S Audit Program Allowable/Unallowable Costs — ARPA</t>
+          <t>AUD-101S Overall Audit Program — Uniform Guidance</t>
         </is>
       </c>
       <c r="C136" s="3" t="inlineStr">
@@ -4048,19 +3932,15 @@
       </c>
       <c r="D136" s="3" t="inlineStr">
         <is>
-          <t>Allowability testing — subsidiary of controls program</t>
+          <t>SA master audit program roadmap</t>
         </is>
       </c>
       <c r="E136" s="3" t="inlineStr">
         <is>
-          <t>8101, 8004</t>
-        </is>
-      </c>
-      <c r="F136" s="3" t="inlineStr">
-        <is>
-          <t>One of these will generate for each direct &amp; material requirement.</t>
-        </is>
-      </c>
+          <t>8000</t>
+        </is>
+      </c>
+      <c r="F136" s="3" t="n"/>
       <c r="G136" s="3" t="inlineStr">
         <is>
           <t>if-single-audit</t>
@@ -4068,19 +3948,19 @@
       </c>
       <c r="H136" s="3" t="inlineStr">
         <is>
-          <t>AUD-801S</t>
+          <t>AUD-101S</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" s="3" t="inlineStr">
         <is>
-          <t>8101.2</t>
+          <t>8001</t>
         </is>
       </c>
       <c r="B137" s="3" t="inlineStr">
         <is>
-          <t>AUD-814S Audit Program Reporting — ARPA</t>
+          <t>KBA-101S Overall Uniform Guidance Compliance Audit Strategy</t>
         </is>
       </c>
       <c r="C137" s="3" t="inlineStr">
@@ -4090,12 +3970,12 @@
       </c>
       <c r="D137" s="3" t="inlineStr">
         <is>
-          <t>Reporting requirement compliance testing</t>
+          <t>SA audit strategy</t>
         </is>
       </c>
       <c r="E137" s="3" t="inlineStr">
         <is>
-          <t>8101, 8004</t>
+          <t>8000, 8000.1</t>
         </is>
       </c>
       <c r="F137" s="3" t="n"/>
@@ -4106,19 +3986,19 @@
       </c>
       <c r="H137" s="3" t="inlineStr">
         <is>
-          <t>AUD-814S</t>
+          <t>KBA-101S</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" s="3" t="inlineStr">
         <is>
-          <t>8101.3</t>
+          <t>8001.1</t>
         </is>
       </c>
       <c r="B138" s="3" t="inlineStr">
         <is>
-          <t>AUD-802S Audit Program Government — ARPA</t>
+          <t>KBA-302S Understanding Entity and Its Program Environment</t>
         </is>
       </c>
       <c r="C138" s="3" t="inlineStr">
@@ -4128,12 +4008,12 @@
       </c>
       <c r="D138" s="3" t="inlineStr">
         <is>
-          <t>Government/allowable costs compliance program</t>
+          <t>Entity program environment understanding</t>
         </is>
       </c>
       <c r="E138" s="3" t="inlineStr">
         <is>
-          <t>8101, 8004</t>
+          <t>8001, 0300</t>
         </is>
       </c>
       <c r="F138" s="3" t="n"/>
@@ -4144,19 +4024,19 @@
       </c>
       <c r="H138" s="3" t="inlineStr">
         <is>
-          <t>AUD-802S</t>
+          <t>KBA-302S</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" s="3" t="inlineStr">
         <is>
-          <t>8101.4</t>
+          <t>8001.2</t>
         </is>
       </c>
       <c r="B139" s="3" t="inlineStr">
         <is>
-          <t>AUD-810S Audit Program Period of Performance — ARPA</t>
+          <t>KBA-503S Basis for Assessment of Inherent Risk of Noncompliance</t>
         </is>
       </c>
       <c r="C139" s="3" t="inlineStr">
@@ -4166,12 +4046,12 @@
       </c>
       <c r="D139" s="3" t="inlineStr">
         <is>
-          <t>Period of performance compliance testing</t>
+          <t>IR assessment for compliance</t>
         </is>
       </c>
       <c r="E139" s="3" t="inlineStr">
         <is>
-          <t>8101, 8004</t>
+          <t>8001.1, 0501</t>
         </is>
       </c>
       <c r="F139" s="3" t="n"/>
@@ -4182,19 +4062,19 @@
       </c>
       <c r="H139" s="3" t="inlineStr">
         <is>
-          <t>AUD-810S</t>
+          <t>KBA-503S</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" s="3" t="inlineStr">
         <is>
-          <t>8101.5</t>
+          <t>8002</t>
         </is>
       </c>
       <c r="B140" s="3" t="inlineStr">
         <is>
-          <t>AUD-811S Audit Program Procurement — ARPA</t>
+          <t>KBA-301S Compliance Requirement Materiality</t>
         </is>
       </c>
       <c r="C140" s="3" t="inlineStr">
@@ -4204,12 +4084,12 @@
       </c>
       <c r="D140" s="3" t="inlineStr">
         <is>
-          <t>Procurement compliance testing</t>
+          <t>Materiality at major program and compliance requirement levels</t>
         </is>
       </c>
       <c r="E140" s="3" t="inlineStr">
         <is>
-          <t>8101, 8004</t>
+          <t>0202, 8001</t>
         </is>
       </c>
       <c r="F140" s="3" t="n"/>
@@ -4220,68 +4100,76 @@
       </c>
       <c r="H140" s="3" t="inlineStr">
         <is>
-          <t>AUD-811S</t>
+          <t>KBA-301S</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" s="3" t="inlineStr">
         <is>
-          <t>8102</t>
+          <t>8003</t>
         </is>
       </c>
       <c r="B141" s="3" t="inlineStr">
         <is>
-          <t>Grant Agreements</t>
+          <t>AID-301S Audit Applicability and Major Programs (SA-18)</t>
         </is>
       </c>
       <c r="C141" s="3" t="inlineStr">
         <is>
-          <t>Workpaper</t>
+          <t>KC Form</t>
         </is>
       </c>
       <c r="D141" s="3" t="inlineStr">
         <is>
-          <t>Grant agreement documentation for ARPA award</t>
+          <t>Major program determination — drives which 8100+ sections exist</t>
         </is>
       </c>
       <c r="E141" s="3" t="inlineStr">
         <is>
-          <t>Client</t>
-        </is>
-      </c>
-      <c r="F141" s="3" t="n"/>
+          <t>2201 (SEFA), 8002</t>
+        </is>
+      </c>
+      <c r="F141" s="3" t="inlineStr">
+        <is>
+          <t>Complete before KBA-502S; drives risk scope</t>
+        </is>
+      </c>
       <c r="G141" s="3" t="inlineStr">
         <is>
           <t>if-single-audit</t>
         </is>
       </c>
-      <c r="H141" s="3" t="inlineStr"/>
+      <c r="H141" s="3" t="inlineStr">
+        <is>
+          <t>AID-301S</t>
+        </is>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="3" t="inlineStr">
         <is>
-          <t>8103</t>
+          <t>8004</t>
         </is>
       </c>
       <c r="B142" s="3" t="inlineStr">
         <is>
-          <t>SA Expenditures Testing</t>
+          <t>KBA-502S Summary of Risk Assessments — Noncompliance</t>
         </is>
       </c>
       <c r="C142" s="3" t="inlineStr">
         <is>
-          <t>Workpaper</t>
+          <t>KC Form</t>
         </is>
       </c>
       <c r="D142" s="3" t="inlineStr">
         <is>
-          <t>Lead expenditure sampling/testing workpaper for ARPA</t>
+          <t>Compliance risk summary by requirement; living document</t>
         </is>
       </c>
       <c r="E142" s="3" t="inlineStr">
         <is>
-          <t>8100.1, 8101.1</t>
+          <t>8003, 8001.2</t>
         </is>
       </c>
       <c r="F142" s="3" t="n"/>
@@ -4290,32 +4178,36 @@
           <t>if-single-audit</t>
         </is>
       </c>
-      <c r="H142" s="3" t="inlineStr"/>
+      <c r="H142" s="3" t="inlineStr">
+        <is>
+          <t>KBA-502S</t>
+        </is>
+      </c>
     </row>
     <row r="143">
       <c r="A143" s="3" t="inlineStr">
         <is>
-          <t>8104</t>
+          <t>8005</t>
         </is>
       </c>
       <c r="B143" s="3" t="inlineStr">
         <is>
-          <t>21.027 Activities/Matching Testing</t>
+          <t>KBA-102S Uniform Guidance Compliance Audit Significant Matters</t>
         </is>
       </c>
       <c r="C143" s="3" t="inlineStr">
         <is>
-          <t>Workpaper</t>
+          <t>KC Form</t>
         </is>
       </c>
       <c r="D143" s="3" t="inlineStr">
         <is>
-          <t>Activities and matching requirement testing workpaper</t>
+          <t>SA significant matters/completion document</t>
         </is>
       </c>
       <c r="E143" s="3" t="inlineStr">
         <is>
-          <t>8101.3</t>
+          <t>All 8100+ complete</t>
         </is>
       </c>
       <c r="F143" s="3" t="n"/>
@@ -4324,32 +4216,36 @@
           <t>if-single-audit</t>
         </is>
       </c>
-      <c r="H143" s="3" t="inlineStr"/>
+      <c r="H143" s="3" t="inlineStr">
+        <is>
+          <t>KBA-102S</t>
+        </is>
+      </c>
     </row>
     <row r="144">
       <c r="A144" s="3" t="inlineStr">
         <is>
-          <t>8105</t>
+          <t>8006</t>
         </is>
       </c>
       <c r="B144" s="3" t="inlineStr">
         <is>
-          <t>21.027 Subrecipient/Period Testing</t>
+          <t>KCO-001 Single Audit Title Overview</t>
         </is>
       </c>
       <c r="C144" s="3" t="inlineStr">
         <is>
-          <t>Workpaper</t>
+          <t>KC Form</t>
         </is>
       </c>
       <c r="D144" s="3" t="inlineStr">
         <is>
-          <t>Subrecipient monitoring and period of performance testing</t>
+          <t>Knowledge Coach SA overview reference</t>
         </is>
       </c>
       <c r="E144" s="3" t="inlineStr">
         <is>
-          <t>8101.4</t>
+          <t>8000</t>
         </is>
       </c>
       <c r="F144" s="3" t="n"/>
@@ -4358,51 +4254,63 @@
           <t>if-single-audit</t>
         </is>
       </c>
-      <c r="H144" s="3" t="inlineStr"/>
+      <c r="H144" s="3" t="inlineStr">
+        <is>
+          <t>KCO-001</t>
+        </is>
+      </c>
     </row>
     <row r="145">
       <c r="A145" s="3" t="inlineStr">
         <is>
-          <t>8106–8109</t>
+          <t>8006.1</t>
         </is>
       </c>
       <c r="B145" s="3" t="inlineStr">
         <is>
-          <t>(Reserved — Additional SA Testing Workpapers)</t>
+          <t>KBA-401S Understanding Entity-Level Controls over Compliance</t>
         </is>
       </c>
       <c r="C145" s="3" t="inlineStr">
         <is>
-          <t>Workpaper</t>
+          <t>KC Form</t>
         </is>
       </c>
       <c r="D145" s="3" t="inlineStr">
         <is>
-          <t>Reserved slots for additional program-specific compliance testing workpapers as needed</t>
+          <t>Entity-level controls specific to federal compliance</t>
         </is>
       </c>
       <c r="E145" s="3" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F145" s="3" t="n"/>
+          <t>0400, 8001.1</t>
+        </is>
+      </c>
+      <c r="F145" s="3" t="inlineStr">
+        <is>
+          <t>8-page form — separate from FS KBA-401</t>
+        </is>
+      </c>
       <c r="G145" s="3" t="inlineStr">
         <is>
           <t>if-single-audit</t>
         </is>
       </c>
-      <c r="H145" s="3" t="inlineStr"/>
+      <c r="H145" s="3" t="inlineStr">
+        <is>
+          <t>KBA-401S</t>
+        </is>
+      </c>
     </row>
     <row r="146">
       <c r="A146" s="3" t="inlineStr">
         <is>
-          <t>8110</t>
+          <t>8006.2</t>
         </is>
       </c>
       <c r="B146" s="3" t="inlineStr">
         <is>
-          <t>KBA-103S Summary and Eval of Noncompliance — ARPA</t>
+          <t>AID-401S Understanding General IT Controls over Compliance</t>
         </is>
       </c>
       <c r="C146" s="3" t="inlineStr">
@@ -4412,19 +4320,15 @@
       </c>
       <c r="D146" s="3" t="inlineStr">
         <is>
-          <t>Noncompliance summary for ARPA; complete after all testing; one per major program</t>
+          <t>IT controls over compliance programs</t>
         </is>
       </c>
       <c r="E146" s="3" t="inlineStr">
         <is>
-          <t>8103–8105 complete</t>
-        </is>
-      </c>
-      <c r="F146" s="3" t="inlineStr">
-        <is>
-          <t>Last substantive SA paper before documentation checklist</t>
-        </is>
-      </c>
+          <t>0400.1, 8006.1</t>
+        </is>
+      </c>
+      <c r="F146" s="3" t="n"/>
       <c r="G146" s="3" t="inlineStr">
         <is>
           <t>if-single-audit</t>
@@ -4432,7 +4336,7 @@
       </c>
       <c r="H146" s="3" t="inlineStr">
         <is>
-          <t>KBA-103S</t>
+          <t>AID-401S</t>
         </is>
       </c>
     </row>
@@ -4449,7 +4353,7 @@
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
         <is>
-          <t>SECTION 90 — PERM FILE</t>
+          <t>SECTION 81 — SINGLE AUDIT: ARPA (CFDA 21.027)</t>
         </is>
       </c>
       <c r="B148" s="3" t="n"/>
@@ -4463,102 +4367,692 @@
     <row r="149">
       <c r="A149" s="3" t="inlineStr">
         <is>
-          <t>9000</t>
+          <t>8100</t>
         </is>
       </c>
       <c r="B149" s="3" t="inlineStr">
         <is>
-          <t>Perm File</t>
+          <t>KBA-400S Identification of D&amp;M Compliance Requirements — ARPA</t>
         </is>
       </c>
       <c r="C149" s="3" t="inlineStr">
         <is>
-          <t>Folder</t>
+          <t>KC Form</t>
         </is>
       </c>
       <c r="D149" s="3" t="inlineStr">
         <is>
-          <t>Permanent file</t>
+          <t>Identifies direct and material compliance requirements; complete before programs</t>
         </is>
       </c>
       <c r="E149" s="3" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F149" s="3" t="n"/>
-      <c r="G149" s="3" t="inlineStr"/>
-      <c r="H149" s="3" t="inlineStr"/>
+          <t>8003, 8001.1</t>
+        </is>
+      </c>
+      <c r="F149" s="3" t="inlineStr">
+        <is>
+          <t>CRITICAL — complete before 8101+</t>
+        </is>
+      </c>
+      <c r="G149" s="3" t="inlineStr">
+        <is>
+          <t>if-single-audit</t>
+        </is>
+      </c>
+      <c r="H149" s="3" t="inlineStr">
+        <is>
+          <t>KBA-400S</t>
+        </is>
+      </c>
     </row>
     <row r="150">
       <c r="A150" s="3" t="inlineStr">
         <is>
-          <t>9100</t>
+          <t>8100.1</t>
         </is>
       </c>
       <c r="B150" s="3" t="inlineStr">
         <is>
-          <t>Org Docs</t>
+          <t>AID-303S Determining Compliance Audit Materiality (SA-18)</t>
         </is>
       </c>
       <c r="C150" s="3" t="inlineStr">
         <is>
-          <t>Folder</t>
+          <t>Excel</t>
         </is>
       </c>
       <c r="D150" s="3" t="inlineStr">
         <is>
-          <t>Organizational documents</t>
+          <t>Compliance audit materiality worksheet for ARPA</t>
         </is>
       </c>
       <c r="E150" s="3" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F150" s="3" t="n"/>
-      <c r="G150" s="3" t="inlineStr"/>
-      <c r="H150" s="3" t="inlineStr"/>
+          <t>8002, 8100</t>
+        </is>
+      </c>
+      <c r="F150" s="3" t="inlineStr">
+        <is>
+          <t>Excel workpaper</t>
+        </is>
+      </c>
+      <c r="G150" s="3" t="inlineStr">
+        <is>
+          <t>if-single-audit</t>
+        </is>
+      </c>
+      <c r="H150" s="3" t="inlineStr">
+        <is>
+          <t>AID-303S</t>
+        </is>
+      </c>
     </row>
     <row r="151">
       <c r="A151" s="3" t="inlineStr">
         <is>
+          <t>8100.2</t>
+        </is>
+      </c>
+      <c r="B151" s="3" t="inlineStr">
+        <is>
+          <t>Compliance Supplement — ARPA 21.027 (Highlighted)</t>
+        </is>
+      </c>
+      <c r="C151" s="3" t="inlineStr">
+        <is>
+          <t>Support Doc</t>
+        </is>
+      </c>
+      <c r="D151" s="3" t="inlineStr">
+        <is>
+          <t>Applicable compliance supplement with requirements highlighted</t>
+        </is>
+      </c>
+      <c r="E151" s="3" t="inlineStr">
+        <is>
+          <t>8100</t>
+        </is>
+      </c>
+      <c r="F151" s="3" t="inlineStr">
+        <is>
+          <t>Highlight applicable requirements before testing</t>
+        </is>
+      </c>
+      <c r="G151" s="3" t="inlineStr">
+        <is>
+          <t>if-single-audit</t>
+        </is>
+      </c>
+      <c r="H151" s="3" t="inlineStr"/>
+    </row>
+    <row r="152">
+      <c r="A152" s="3" t="inlineStr">
+        <is>
+          <t>8101</t>
+        </is>
+      </c>
+      <c r="B152" s="3" t="inlineStr">
+        <is>
+          <t>AUD-701S Audit Program Designing Tests of Controls over Compliance — ARPA</t>
+        </is>
+      </c>
+      <c r="C152" s="3" t="inlineStr">
+        <is>
+          <t>KC Form</t>
+        </is>
+      </c>
+      <c r="D152" s="3" t="inlineStr">
+        <is>
+          <t>Lead controls testing program for ARPA compliance</t>
+        </is>
+      </c>
+      <c r="E152" s="3" t="inlineStr">
+        <is>
+          <t>8006.1, 8100</t>
+        </is>
+      </c>
+      <c r="F152" s="3" t="n"/>
+      <c r="G152" s="3" t="inlineStr">
+        <is>
+          <t>if-single-audit</t>
+        </is>
+      </c>
+      <c r="H152" s="3" t="inlineStr">
+        <is>
+          <t>AUD-701S</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" s="3" t="inlineStr">
+        <is>
+          <t>8101.1</t>
+        </is>
+      </c>
+      <c r="B153" s="3" t="inlineStr">
+        <is>
+          <t>AUD-801S Audit Program Allowable/Unallowable Costs — ARPA</t>
+        </is>
+      </c>
+      <c r="C153" s="3" t="inlineStr">
+        <is>
+          <t>KC Form</t>
+        </is>
+      </c>
+      <c r="D153" s="3" t="inlineStr">
+        <is>
+          <t>Allowability testing — subsidiary of controls program</t>
+        </is>
+      </c>
+      <c r="E153" s="3" t="inlineStr">
+        <is>
+          <t>8101, 8004</t>
+        </is>
+      </c>
+      <c r="F153" s="3" t="inlineStr">
+        <is>
+          <t>One of these will generate for each direct &amp; material requirement.</t>
+        </is>
+      </c>
+      <c r="G153" s="3" t="inlineStr">
+        <is>
+          <t>if-single-audit</t>
+        </is>
+      </c>
+      <c r="H153" s="3" t="inlineStr">
+        <is>
+          <t>AUD-801S</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" s="3" t="inlineStr">
+        <is>
+          <t>8101.2</t>
+        </is>
+      </c>
+      <c r="B154" s="3" t="inlineStr">
+        <is>
+          <t>AUD-814S Audit Program Reporting — ARPA</t>
+        </is>
+      </c>
+      <c r="C154" s="3" t="inlineStr">
+        <is>
+          <t>KC Form</t>
+        </is>
+      </c>
+      <c r="D154" s="3" t="inlineStr">
+        <is>
+          <t>Reporting requirement compliance testing</t>
+        </is>
+      </c>
+      <c r="E154" s="3" t="inlineStr">
+        <is>
+          <t>8101, 8004</t>
+        </is>
+      </c>
+      <c r="F154" s="3" t="n"/>
+      <c r="G154" s="3" t="inlineStr">
+        <is>
+          <t>if-single-audit</t>
+        </is>
+      </c>
+      <c r="H154" s="3" t="inlineStr">
+        <is>
+          <t>AUD-814S</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" s="3" t="inlineStr">
+        <is>
+          <t>8101.3</t>
+        </is>
+      </c>
+      <c r="B155" s="3" t="inlineStr">
+        <is>
+          <t>AUD-802S Audit Program Government — ARPA</t>
+        </is>
+      </c>
+      <c r="C155" s="3" t="inlineStr">
+        <is>
+          <t>KC Form</t>
+        </is>
+      </c>
+      <c r="D155" s="3" t="inlineStr">
+        <is>
+          <t>Government/allowable costs compliance program</t>
+        </is>
+      </c>
+      <c r="E155" s="3" t="inlineStr">
+        <is>
+          <t>8101, 8004</t>
+        </is>
+      </c>
+      <c r="F155" s="3" t="n"/>
+      <c r="G155" s="3" t="inlineStr">
+        <is>
+          <t>if-single-audit</t>
+        </is>
+      </c>
+      <c r="H155" s="3" t="inlineStr">
+        <is>
+          <t>AUD-802S</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" s="3" t="inlineStr">
+        <is>
+          <t>8101.4</t>
+        </is>
+      </c>
+      <c r="B156" s="3" t="inlineStr">
+        <is>
+          <t>AUD-810S Audit Program Period of Performance — ARPA</t>
+        </is>
+      </c>
+      <c r="C156" s="3" t="inlineStr">
+        <is>
+          <t>KC Form</t>
+        </is>
+      </c>
+      <c r="D156" s="3" t="inlineStr">
+        <is>
+          <t>Period of performance compliance testing</t>
+        </is>
+      </c>
+      <c r="E156" s="3" t="inlineStr">
+        <is>
+          <t>8101, 8004</t>
+        </is>
+      </c>
+      <c r="F156" s="3" t="n"/>
+      <c r="G156" s="3" t="inlineStr">
+        <is>
+          <t>if-single-audit</t>
+        </is>
+      </c>
+      <c r="H156" s="3" t="inlineStr">
+        <is>
+          <t>AUD-810S</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" s="3" t="inlineStr">
+        <is>
+          <t>8101.5</t>
+        </is>
+      </c>
+      <c r="B157" s="3" t="inlineStr">
+        <is>
+          <t>AUD-811S Audit Program Procurement — ARPA</t>
+        </is>
+      </c>
+      <c r="C157" s="3" t="inlineStr">
+        <is>
+          <t>KC Form</t>
+        </is>
+      </c>
+      <c r="D157" s="3" t="inlineStr">
+        <is>
+          <t>Procurement compliance testing</t>
+        </is>
+      </c>
+      <c r="E157" s="3" t="inlineStr">
+        <is>
+          <t>8101, 8004</t>
+        </is>
+      </c>
+      <c r="F157" s="3" t="n"/>
+      <c r="G157" s="3" t="inlineStr">
+        <is>
+          <t>if-single-audit</t>
+        </is>
+      </c>
+      <c r="H157" s="3" t="inlineStr">
+        <is>
+          <t>AUD-811S</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" s="3" t="inlineStr">
+        <is>
+          <t>8102</t>
+        </is>
+      </c>
+      <c r="B158" s="3" t="inlineStr">
+        <is>
+          <t>Grant Agreements</t>
+        </is>
+      </c>
+      <c r="C158" s="3" t="inlineStr">
+        <is>
+          <t>Workpaper</t>
+        </is>
+      </c>
+      <c r="D158" s="3" t="inlineStr">
+        <is>
+          <t>Grant agreement documentation for ARPA award</t>
+        </is>
+      </c>
+      <c r="E158" s="3" t="inlineStr">
+        <is>
+          <t>Client</t>
+        </is>
+      </c>
+      <c r="F158" s="3" t="n"/>
+      <c r="G158" s="3" t="inlineStr">
+        <is>
+          <t>if-single-audit</t>
+        </is>
+      </c>
+      <c r="H158" s="3" t="inlineStr"/>
+    </row>
+    <row r="159">
+      <c r="A159" s="3" t="inlineStr">
+        <is>
+          <t>8103</t>
+        </is>
+      </c>
+      <c r="B159" s="3" t="inlineStr">
+        <is>
+          <t>SA Expenditures Testing</t>
+        </is>
+      </c>
+      <c r="C159" s="3" t="inlineStr">
+        <is>
+          <t>Workpaper</t>
+        </is>
+      </c>
+      <c r="D159" s="3" t="inlineStr">
+        <is>
+          <t>Lead expenditure sampling/testing workpaper for ARPA</t>
+        </is>
+      </c>
+      <c r="E159" s="3" t="inlineStr">
+        <is>
+          <t>8100.1, 8101.1</t>
+        </is>
+      </c>
+      <c r="F159" s="3" t="n"/>
+      <c r="G159" s="3" t="inlineStr">
+        <is>
+          <t>if-single-audit</t>
+        </is>
+      </c>
+      <c r="H159" s="3" t="inlineStr"/>
+    </row>
+    <row r="160">
+      <c r="A160" s="3" t="inlineStr">
+        <is>
+          <t>8104</t>
+        </is>
+      </c>
+      <c r="B160" s="3" t="inlineStr">
+        <is>
+          <t>21.027 Activities/Matching Testing</t>
+        </is>
+      </c>
+      <c r="C160" s="3" t="inlineStr">
+        <is>
+          <t>Workpaper</t>
+        </is>
+      </c>
+      <c r="D160" s="3" t="inlineStr">
+        <is>
+          <t>Activities and matching requirement testing workpaper</t>
+        </is>
+      </c>
+      <c r="E160" s="3" t="inlineStr">
+        <is>
+          <t>8101.3</t>
+        </is>
+      </c>
+      <c r="F160" s="3" t="n"/>
+      <c r="G160" s="3" t="inlineStr">
+        <is>
+          <t>if-single-audit</t>
+        </is>
+      </c>
+      <c r="H160" s="3" t="inlineStr"/>
+    </row>
+    <row r="161">
+      <c r="A161" s="3" t="inlineStr">
+        <is>
+          <t>8105</t>
+        </is>
+      </c>
+      <c r="B161" s="3" t="inlineStr">
+        <is>
+          <t>21.027 Subrecipient/Period Testing</t>
+        </is>
+      </c>
+      <c r="C161" s="3" t="inlineStr">
+        <is>
+          <t>Workpaper</t>
+        </is>
+      </c>
+      <c r="D161" s="3" t="inlineStr">
+        <is>
+          <t>Subrecipient monitoring and period of performance testing</t>
+        </is>
+      </c>
+      <c r="E161" s="3" t="inlineStr">
+        <is>
+          <t>8101.4</t>
+        </is>
+      </c>
+      <c r="F161" s="3" t="n"/>
+      <c r="G161" s="3" t="inlineStr">
+        <is>
+          <t>if-single-audit</t>
+        </is>
+      </c>
+      <c r="H161" s="3" t="inlineStr"/>
+    </row>
+    <row r="162">
+      <c r="A162" s="3" t="inlineStr">
+        <is>
+          <t>8106–8109</t>
+        </is>
+      </c>
+      <c r="B162" s="3" t="inlineStr">
+        <is>
+          <t>(Reserved — Additional SA Testing Workpapers)</t>
+        </is>
+      </c>
+      <c r="C162" s="3" t="inlineStr">
+        <is>
+          <t>Workpaper</t>
+        </is>
+      </c>
+      <c r="D162" s="3" t="inlineStr">
+        <is>
+          <t>Reserved slots for additional program-specific compliance testing workpapers as needed</t>
+        </is>
+      </c>
+      <c r="E162" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F162" s="3" t="n"/>
+      <c r="G162" s="3" t="inlineStr">
+        <is>
+          <t>if-single-audit</t>
+        </is>
+      </c>
+      <c r="H162" s="3" t="inlineStr"/>
+    </row>
+    <row r="163">
+      <c r="A163" s="3" t="inlineStr">
+        <is>
+          <t>8110</t>
+        </is>
+      </c>
+      <c r="B163" s="3" t="inlineStr">
+        <is>
+          <t>KBA-103S Summary and Eval of Noncompliance — ARPA</t>
+        </is>
+      </c>
+      <c r="C163" s="3" t="inlineStr">
+        <is>
+          <t>KC Form</t>
+        </is>
+      </c>
+      <c r="D163" s="3" t="inlineStr">
+        <is>
+          <t>Noncompliance summary for ARPA; complete after all testing; one per major program</t>
+        </is>
+      </c>
+      <c r="E163" s="3" t="inlineStr">
+        <is>
+          <t>8103–8105 complete</t>
+        </is>
+      </c>
+      <c r="F163" s="3" t="inlineStr">
+        <is>
+          <t>Last substantive SA paper before documentation checklist</t>
+        </is>
+      </c>
+      <c r="G163" s="3" t="inlineStr">
+        <is>
+          <t>if-single-audit</t>
+        </is>
+      </c>
+      <c r="H163" s="3" t="inlineStr">
+        <is>
+          <t>KBA-103S</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" s="3" t="n"/>
+      <c r="B164" s="3" t="n"/>
+      <c r="C164" s="3" t="n"/>
+      <c r="D164" s="3" t="n"/>
+      <c r="E164" s="3" t="n"/>
+      <c r="F164" s="3" t="n"/>
+      <c r="G164" s="3" t="n"/>
+      <c r="H164" s="3" t="n"/>
+    </row>
+    <row r="165">
+      <c r="A165" s="2" t="inlineStr">
+        <is>
+          <t>SECTION 90 — PERM FILE</t>
+        </is>
+      </c>
+      <c r="B165" s="3" t="n"/>
+      <c r="C165" s="3" t="n"/>
+      <c r="D165" s="3" t="n"/>
+      <c r="E165" s="3" t="n"/>
+      <c r="F165" s="3" t="n"/>
+      <c r="G165" s="3" t="n"/>
+      <c r="H165" s="3" t="n"/>
+    </row>
+    <row r="166">
+      <c r="A166" s="3" t="inlineStr">
+        <is>
+          <t>9000</t>
+        </is>
+      </c>
+      <c r="B166" s="3" t="inlineStr">
+        <is>
+          <t>Perm File</t>
+        </is>
+      </c>
+      <c r="C166" s="3" t="inlineStr">
+        <is>
+          <t>Folder</t>
+        </is>
+      </c>
+      <c r="D166" s="3" t="inlineStr">
+        <is>
+          <t>Permanent file</t>
+        </is>
+      </c>
+      <c r="E166" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F166" s="3" t="n"/>
+      <c r="G166" s="3" t="inlineStr"/>
+      <c r="H166" s="3" t="inlineStr"/>
+    </row>
+    <row r="167">
+      <c r="A167" s="3" t="inlineStr">
+        <is>
+          <t>9100</t>
+        </is>
+      </c>
+      <c r="B167" s="3" t="inlineStr">
+        <is>
+          <t>Org Docs</t>
+        </is>
+      </c>
+      <c r="C167" s="3" t="inlineStr">
+        <is>
+          <t>Folder</t>
+        </is>
+      </c>
+      <c r="D167" s="3" t="inlineStr">
+        <is>
+          <t>Organizational documents</t>
+        </is>
+      </c>
+      <c r="E167" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F167" s="3" t="n"/>
+      <c r="G167" s="3" t="inlineStr"/>
+      <c r="H167" s="3" t="inlineStr"/>
+    </row>
+    <row r="168">
+      <c r="A168" s="3" t="inlineStr">
+        <is>
           <t>9200</t>
         </is>
       </c>
-      <c r="B151" s="3" t="inlineStr">
+      <c r="B168" s="3" t="inlineStr">
         <is>
           <t>Policies</t>
         </is>
       </c>
-      <c r="C151" s="3" t="inlineStr">
+      <c r="C168" s="3" t="inlineStr">
         <is>
           <t>Folder</t>
         </is>
       </c>
-      <c r="D151" s="3" t="inlineStr">
+      <c r="D168" s="3" t="inlineStr">
         <is>
           <t>Policy documents</t>
         </is>
       </c>
-      <c r="E151" s="3" t="inlineStr">
+      <c r="E168" s="3" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="F151" s="3" t="n"/>
-      <c r="G151" s="3" t="inlineStr"/>
-      <c r="H151" s="3" t="inlineStr"/>
-    </row>
-    <row r="152">
-      <c r="A152" s="3" t="n"/>
-      <c r="B152" s="3" t="n"/>
-      <c r="C152" s="3" t="n"/>
-      <c r="D152" s="3" t="n"/>
-      <c r="E152" s="3" t="n"/>
-      <c r="F152" s="3" t="n"/>
-      <c r="G152" s="3" t="n"/>
-      <c r="H152" s="3" t="n"/>
+      <c r="F168" s="3" t="n"/>
+      <c r="G168" s="3" t="inlineStr"/>
+      <c r="H168" s="3" t="inlineStr"/>
+    </row>
+    <row r="169">
+      <c r="A169" s="3" t="n"/>
+      <c r="B169" s="3" t="n"/>
+      <c r="C169" s="3" t="n"/>
+      <c r="D169" s="3" t="n"/>
+      <c r="E169" s="3" t="n"/>
+      <c r="F169" s="3" t="n"/>
+      <c r="G169" s="3" t="n"/>
+      <c r="H169" s="3" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>